<commit_message>
Fossil: 6 core SKUs always 12 weeks cover, fix string cols, zero qty when SOH=0
</commit_message>
<xml_diff>
--- a/data/input/Fossil Replenishment/Fossil Replenishment.xlsx
+++ b/data/input/Fossil Replenishment/Fossil Replenishment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Fossil Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD860362-0F4E-4DE6-9A82-898793CE9777}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D0C406E-7606-4000-99F8-756B018A1E5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6662473D-6E1F-42FD-999B-28162E22D4B5}"/>
   </bookViews>
@@ -4521,7 +4521,7 @@
         <v>1069</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H11" s="8" t="s">
         <v>12</v>
@@ -8346,7 +8346,7 @@
         <v>1070</v>
       </c>
       <c r="G86" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H86" s="8" t="s">
         <v>12</v>
@@ -31566,7 +31566,6 @@
       <c r="T766" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T374" xr:uid="{AF55B7BF-85DC-4082-9A73-200B4D79A598}"/>
   <conditionalFormatting sqref="A1:B1">
     <cfRule type="duplicateValues" dxfId="5" priority="5"/>
     <cfRule type="duplicateValues" dxfId="4" priority="6"/>

</xml_diff>

<commit_message>
Update Fossil master and In-Transit/Open PO data
</commit_message>
<xml_diff>
--- a/data/input/Fossil Replenishment/Fossil Replenishment.xlsx
+++ b/data/input/Fossil Replenishment/Fossil Replenishment.xlsx
@@ -32167,15 +32167,15 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:T384" xr:uid="{AF55B7BF-85DC-4082-9A73-200B4D79A598}"/>
+  <conditionalFormatting sqref="A1:B1">
+    <cfRule type="duplicateValues" dxfId="5" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="14"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="5" priority="7"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="3" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="10"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:B1">
-    <cfRule type="duplicateValues" dxfId="1" priority="13"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="10"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Data: refresh full input folder — weekly data pipeline catch-up
Inventory snapshots, ledgers, Amazon FBA inventory, replenishment
masters, sku_master, weekly sales — all refreshed in one push so input/
is fully in sync.

  - Inventory_snapshot_{WM, audio_array, tonor, nexlev}.xlsx
  - inventory_amazon_{WM, audio_array, nexlev}.csv
  - inventory_ledger_{Audio Array, WM, nexlev}.csv
  - replenishment_master_nexlev.xlsx
  - sku_master.xlsx
  - weekly_sales_snapshot.csv
  - Fossil Replenishment/Fossil Replenishment.xlsx
  - Fossil Replenishment/inventory_ledger_fossil.csv
  - Blinkit/Cluster.xlsx + Serving Cities.xlsx (new untracked)

Audit reports 2 EOL SKUs (FBK79569 / LE-06, FBK79685 / LE-08) in the
Nexlev + Viomi masters that aren't in sku_master — these were flagged
EOL by user and intentionally skipped. WARN expected, not a regression.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Fossil Replenishment/Fossil Replenishment.xlsx
+++ b/data/input/Fossil Replenishment/Fossil Replenishment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Fossil Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3302EB5-14A2-4A41-A106-F49943D5FEA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41DD4EE8-2D85-43AC-823E-B99764E8B6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6662473D-6E1F-42FD-999B-28162E22D4B5}"/>
   </bookViews>
@@ -4800,7 +4800,7 @@
         <v>1068</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H9" s="8" t="s">
         <v>12</v>
@@ -4851,7 +4851,7 @@
         <v>1068</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H10" s="8" t="s">
         <v>12</v>
@@ -6279,7 +6279,7 @@
         <v>1068</v>
       </c>
       <c r="G38" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H38" s="8" t="s">
         <v>12</v>
@@ -7350,7 +7350,7 @@
         <v>1068</v>
       </c>
       <c r="G59" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H59" s="8" t="s">
         <v>13</v>
@@ -7656,7 +7656,7 @@
         <v>1069</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H65" s="8" t="s">
         <v>12</v>
@@ -8166,7 +8166,7 @@
         <v>1068</v>
       </c>
       <c r="G75" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H75" s="8" t="s">
         <v>13</v>
@@ -8217,7 +8217,7 @@
         <v>1069</v>
       </c>
       <c r="G76" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H76" s="8" t="s">
         <v>13</v>
@@ -8727,7 +8727,7 @@
         <v>1068</v>
       </c>
       <c r="G86" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H86" s="8" t="s">
         <v>12</v>
@@ -8982,7 +8982,7 @@
         <v>1069</v>
       </c>
       <c r="G91" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H91" s="8" t="s">
         <v>12</v>
@@ -9084,7 +9084,7 @@
         <v>1068</v>
       </c>
       <c r="G93" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H93" s="8" t="s">
         <v>13</v>
@@ -9135,7 +9135,7 @@
         <v>1068</v>
       </c>
       <c r="G94" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H94" s="8" t="s">
         <v>12</v>
@@ -9594,7 +9594,7 @@
         <v>1068</v>
       </c>
       <c r="G103" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H103" s="8" t="s">
         <v>15</v>
@@ -10614,7 +10614,7 @@
         <v>1068</v>
       </c>
       <c r="G123" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H123" s="8" t="s">
         <v>14</v>
@@ -10767,7 +10767,7 @@
         <v>1068</v>
       </c>
       <c r="G126" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H126" s="8" t="s">
         <v>17</v>
@@ -11022,7 +11022,7 @@
         <v>1068</v>
       </c>
       <c r="G131" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H131" s="8" t="s">
         <v>14</v>
@@ -11226,7 +11226,7 @@
         <v>1069</v>
       </c>
       <c r="G135" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H135" s="8" t="s">
         <v>15</v>
@@ -11481,7 +11481,7 @@
         <v>1069</v>
       </c>
       <c r="G140" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H140" s="8" t="s">
         <v>15</v>
@@ -11940,7 +11940,7 @@
         <v>1068</v>
       </c>
       <c r="G149" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H149" s="8" t="s">
         <v>12</v>
@@ -11991,7 +11991,7 @@
         <v>1068</v>
       </c>
       <c r="G150" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H150" s="8" t="s">
         <v>12</v>
@@ -12144,7 +12144,7 @@
         <v>1068</v>
       </c>
       <c r="G153" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H153" s="8" t="s">
         <v>13</v>
@@ -12297,7 +12297,7 @@
         <v>1068</v>
       </c>
       <c r="G156" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H156" s="8" t="s">
         <v>15</v>
@@ -12450,7 +12450,7 @@
         <v>1068</v>
       </c>
       <c r="G159" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H159" s="8" t="s">
         <v>15</v>
@@ -12603,7 +12603,7 @@
         <v>1069</v>
       </c>
       <c r="G162" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H162" s="8" t="s">
         <v>13</v>
@@ -12807,7 +12807,7 @@
         <v>1068</v>
       </c>
       <c r="G166" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H166" s="8" t="s">
         <v>14</v>
@@ -13011,7 +13011,7 @@
         <v>1068</v>
       </c>
       <c r="G170" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H170" s="8" t="s">
         <v>14</v>
@@ -14490,7 +14490,7 @@
         <v>1068</v>
       </c>
       <c r="G199" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H199" s="8" t="s">
         <v>14</v>
@@ -14592,7 +14592,7 @@
         <v>1068</v>
       </c>
       <c r="G201" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H201" s="8" t="s">
         <v>12</v>
@@ -14745,7 +14745,7 @@
         <v>1068</v>
       </c>
       <c r="G204" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H204" s="8" t="s">
         <v>13</v>
@@ -14796,7 +14796,7 @@
         <v>1068</v>
       </c>
       <c r="G205" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H205" s="8" t="s">
         <v>16</v>
@@ -15000,7 +15000,7 @@
         <v>1068</v>
       </c>
       <c r="G209" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H209" s="8" t="s">
         <v>12</v>
@@ -15051,7 +15051,7 @@
         <v>1068</v>
       </c>
       <c r="G210" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H210" s="8" t="s">
         <v>13</v>
@@ -15102,7 +15102,7 @@
         <v>1068</v>
       </c>
       <c r="G211" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H211" s="8" t="s">
         <v>12</v>
@@ -15561,7 +15561,7 @@
         <v>1068</v>
       </c>
       <c r="G220" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H220" s="8" t="s">
         <v>16</v>
@@ -15765,7 +15765,7 @@
         <v>1069</v>
       </c>
       <c r="G224" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H224" s="8" t="s">
         <v>13</v>
@@ -16020,7 +16020,7 @@
         <v>1068</v>
       </c>
       <c r="G229" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H229" s="8" t="s">
         <v>15</v>
@@ -16275,7 +16275,7 @@
         <v>1068</v>
       </c>
       <c r="G234" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H234" s="8" t="s">
         <v>15</v>
@@ -16428,7 +16428,7 @@
         <v>1069</v>
       </c>
       <c r="G237" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H237" s="8" t="s">
         <v>12</v>
@@ -16530,7 +16530,7 @@
         <v>1068</v>
       </c>
       <c r="G239" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H239" s="8" t="s">
         <v>15</v>
@@ -16683,7 +16683,7 @@
         <v>1068</v>
       </c>
       <c r="G242" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H242" s="8" t="s">
         <v>12</v>
@@ -16734,7 +16734,7 @@
         <v>1069</v>
       </c>
       <c r="G243" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H243" s="8" t="s">
         <v>15</v>
@@ -16938,7 +16938,7 @@
         <v>1069</v>
       </c>
       <c r="G247" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H247" s="8" t="s">
         <v>13</v>
@@ -17091,7 +17091,7 @@
         <v>1068</v>
       </c>
       <c r="G250" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H250" s="8" t="s">
         <v>12</v>
@@ -17142,7 +17142,7 @@
         <v>1068</v>
       </c>
       <c r="G251" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H251" s="8" t="s">
         <v>14</v>
@@ -17193,7 +17193,7 @@
         <v>1068</v>
       </c>
       <c r="G252" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H252" s="8" t="s">
         <v>14</v>
@@ -17244,7 +17244,7 @@
         <v>1068</v>
       </c>
       <c r="G253" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H253" s="8" t="s">
         <v>14</v>
@@ -17295,7 +17295,7 @@
         <v>1068</v>
       </c>
       <c r="G254" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H254" s="8" t="s">
         <v>14</v>
@@ -17907,7 +17907,7 @@
         <v>1068</v>
       </c>
       <c r="G266" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H266" s="8" t="s">
         <v>14</v>
@@ -18468,7 +18468,7 @@
         <v>1068</v>
       </c>
       <c r="G277" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H277" s="8" t="s">
         <v>13</v>
@@ -18570,7 +18570,7 @@
         <v>1068</v>
       </c>
       <c r="G279" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H279" s="8" t="s">
         <v>13</v>
@@ -19131,7 +19131,7 @@
         <v>1068</v>
       </c>
       <c r="G290" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H290" s="8" t="s">
         <v>14</v>
@@ -19284,7 +19284,7 @@
         <v>1068</v>
       </c>
       <c r="G293" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H293" s="8" t="s">
         <v>12</v>
@@ -19335,7 +19335,7 @@
         <v>1068</v>
       </c>
       <c r="G294" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H294" s="8" t="s">
         <v>12</v>
@@ -19488,7 +19488,7 @@
         <v>1068</v>
       </c>
       <c r="G297" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H297" s="8" t="s">
         <v>17</v>
@@ -19539,7 +19539,7 @@
         <v>1068</v>
       </c>
       <c r="G298" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H298" s="8" t="s">
         <v>14</v>
@@ -20508,7 +20508,7 @@
         <v>1068</v>
       </c>
       <c r="G317" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H317" s="8" t="s">
         <v>12</v>
@@ -22191,7 +22191,7 @@
         <v>1068</v>
       </c>
       <c r="G350" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H350" s="8" t="s">
         <v>13</v>
@@ -22242,7 +22242,7 @@
         <v>1068</v>
       </c>
       <c r="G351" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H351" s="8" t="s">
         <v>15</v>
@@ -22599,7 +22599,7 @@
         <v>1068</v>
       </c>
       <c r="G358" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H358" s="8" t="s">
         <v>13</v>
@@ -23721,7 +23721,7 @@
         <v>1068</v>
       </c>
       <c r="G380" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H380" s="8" t="s">
         <v>12</v>
@@ -23772,7 +23772,7 @@
         <v>1068</v>
       </c>
       <c r="G381" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H381" s="8" t="s">
         <v>17</v>
@@ -24180,7 +24180,7 @@
         <v>1068</v>
       </c>
       <c r="G389" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H389" s="8" t="s">
         <v>12</v>
@@ -24639,7 +24639,7 @@
         <v>418</v>
       </c>
       <c r="G398" s="7" t="s">
-        <v>418</v>
+        <v>1062</v>
       </c>
       <c r="H398" s="7" t="s">
         <v>15</v>
@@ -24791,8 +24791,8 @@
       <c r="F401" s="7" t="s">
         <v>1068</v>
       </c>
-      <c r="G401" s="7" t="s">
-        <v>1061</v>
+      <c r="G401" s="8" t="s">
+        <v>1062</v>
       </c>
       <c r="H401" s="7" t="s">
         <v>15</v>

</xml_diff>

<commit_message>
Fossil refresh 2026-08-11 — Replenishment + In-Transit PO
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/input/Fossil Replenishment/Fossil Replenishment.xlsx
+++ b/data/input/Fossil Replenishment/Fossil Replenishment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Fossil Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92EC844A-B609-4DB7-80EA-459B18E8AE5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA74F32B-9212-4C83-B1CD-CD460BB95FC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6662473D-6E1F-42FD-999B-28162E22D4B5}"/>
   </bookViews>
@@ -4855,23 +4855,23 @@
         <v>12</v>
       </c>
       <c r="I2" s="8">
-        <v>826</v>
+        <v>827</v>
       </c>
       <c r="J2" s="8">
         <v>0</v>
       </c>
       <c r="K2" s="8">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="L2" s="8">
         <v>0</v>
       </c>
       <c r="M2" s="8">
         <f>I2+J2+K2+L2</f>
-        <v>898</v>
+        <v>827</v>
       </c>
       <c r="N2" s="8">
-        <v>1209</v>
+        <v>2191</v>
       </c>
       <c r="O2" s="8"/>
       <c r="P2" s="8"/>
@@ -4906,7 +4906,7 @@
         <v>12</v>
       </c>
       <c r="I3" s="8">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J3" s="8">
         <v>0</v>
@@ -4919,7 +4919,7 @@
       </c>
       <c r="M3" s="8">
         <f t="shared" ref="M3:M66" si="0">I3+J3+K3+L3</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N3" s="8">
         <v>0</v>
@@ -4957,7 +4957,7 @@
         <v>12</v>
       </c>
       <c r="I4" s="8">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="J4" s="8">
         <v>0</v>
@@ -4970,7 +4970,7 @@
       </c>
       <c r="M4" s="8">
         <f t="shared" si="0"/>
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="N4" s="8">
         <v>0</v>
@@ -5008,7 +5008,7 @@
         <v>12</v>
       </c>
       <c r="I5" s="8">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="J5" s="8">
         <v>0</v>
@@ -5017,14 +5017,14 @@
         <v>0</v>
       </c>
       <c r="L5" s="8">
-        <v>0</v>
+        <v>169</v>
       </c>
       <c r="M5" s="8">
         <f t="shared" si="0"/>
-        <v>37</v>
+        <v>189</v>
       </c>
       <c r="N5" s="8">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="O5" s="8"/>
       <c r="P5" s="8"/>
@@ -5059,20 +5059,20 @@
         <v>12</v>
       </c>
       <c r="I6" s="8">
-        <v>869</v>
+        <v>887</v>
       </c>
       <c r="J6" s="8">
         <v>0</v>
       </c>
       <c r="K6" s="8">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="L6" s="8">
         <v>0</v>
       </c>
       <c r="M6" s="8">
         <f t="shared" si="0"/>
-        <v>965</v>
+        <v>887</v>
       </c>
       <c r="N6" s="8">
         <v>1490</v>
@@ -5110,7 +5110,7 @@
         <v>12</v>
       </c>
       <c r="I7" s="8">
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="J7" s="8">
         <v>0</v>
@@ -5123,10 +5123,10 @@
       </c>
       <c r="M7" s="8">
         <f t="shared" si="0"/>
-        <v>173</v>
+        <v>165</v>
       </c>
       <c r="N7" s="8">
-        <v>869</v>
+        <v>575</v>
       </c>
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
@@ -5161,23 +5161,23 @@
         <v>12</v>
       </c>
       <c r="I8" s="8">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="J8" s="8">
         <v>0</v>
       </c>
       <c r="K8" s="8">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="L8" s="8">
-        <v>28</v>
+        <v>0</v>
       </c>
       <c r="M8" s="8">
         <f t="shared" si="0"/>
-        <v>114</v>
+        <v>101</v>
       </c>
       <c r="N8" s="8">
-        <v>318</v>
+        <v>100</v>
       </c>
       <c r="O8" s="8"/>
       <c r="P8" s="8"/>
@@ -5212,7 +5212,7 @@
         <v>12</v>
       </c>
       <c r="I9" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="8">
         <v>0</v>
@@ -5225,7 +5225,7 @@
       </c>
       <c r="M9" s="8">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N9" s="8">
         <v>0</v>
@@ -5314,7 +5314,7 @@
         <v>12</v>
       </c>
       <c r="I11" s="8">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="J11" s="8">
         <v>0</v>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="M11" s="8">
         <f t="shared" si="0"/>
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="N11" s="8">
         <v>0</v>
@@ -5365,7 +5365,7 @@
         <v>12</v>
       </c>
       <c r="I12" s="8">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J12" s="8">
         <v>0</v>
@@ -5378,7 +5378,7 @@
       </c>
       <c r="M12" s="8">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="N12" s="8">
         <v>0</v>
@@ -5416,20 +5416,20 @@
         <v>12</v>
       </c>
       <c r="I13" s="8">
-        <v>229</v>
+        <v>246</v>
       </c>
       <c r="J13" s="8">
         <v>0</v>
       </c>
       <c r="K13" s="8">
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="L13" s="8">
         <v>0</v>
       </c>
       <c r="M13" s="8">
         <f t="shared" si="0"/>
-        <v>277</v>
+        <v>246</v>
       </c>
       <c r="N13" s="8">
         <v>810</v>
@@ -5467,23 +5467,23 @@
         <v>12</v>
       </c>
       <c r="I14" s="8">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="J14" s="8">
         <v>0</v>
       </c>
       <c r="K14" s="8">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L14" s="8">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M14" s="8">
         <f t="shared" si="0"/>
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="N14" s="8">
-        <v>626</v>
+        <v>557</v>
       </c>
       <c r="O14" s="8"/>
       <c r="P14" s="8"/>
@@ -5569,23 +5569,23 @@
         <v>12</v>
       </c>
       <c r="I16" s="8">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="J16" s="8">
         <v>0</v>
       </c>
       <c r="K16" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L16" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M16" s="8">
         <f t="shared" si="0"/>
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N16" s="8">
-        <v>533</v>
+        <v>377</v>
       </c>
       <c r="O16" s="8"/>
       <c r="P16" s="8"/>
@@ -5636,7 +5636,7 @@
         <v>64</v>
       </c>
       <c r="N17" s="8">
-        <v>315</v>
+        <v>285</v>
       </c>
       <c r="O17" s="8"/>
       <c r="P17" s="8"/>
@@ -5671,7 +5671,7 @@
         <v>12</v>
       </c>
       <c r="I18" s="8">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="J18" s="8">
         <v>0</v>
@@ -5684,7 +5684,7 @@
       </c>
       <c r="M18" s="8">
         <f t="shared" si="0"/>
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="N18" s="8">
         <v>0</v>
@@ -5722,7 +5722,7 @@
         <v>13</v>
       </c>
       <c r="I19" s="8">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J19" s="8">
         <v>0</v>
@@ -5735,10 +5735,10 @@
       </c>
       <c r="M19" s="8">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="N19" s="8">
-        <v>405</v>
+        <v>270</v>
       </c>
       <c r="O19" s="8"/>
       <c r="P19" s="8"/>
@@ -5773,7 +5773,7 @@
         <v>14</v>
       </c>
       <c r="I20" s="8">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J20" s="8">
         <v>0</v>
@@ -5782,11 +5782,11 @@
         <v>0</v>
       </c>
       <c r="L20" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M20" s="8">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="N20" s="8">
         <v>0</v>
@@ -5824,7 +5824,7 @@
         <v>13</v>
       </c>
       <c r="I21" s="8">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="J21" s="8">
         <v>0</v>
@@ -5837,7 +5837,7 @@
       </c>
       <c r="M21" s="8">
         <f t="shared" si="0"/>
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="N21" s="8">
         <v>0</v>
@@ -5926,7 +5926,7 @@
         <v>12</v>
       </c>
       <c r="I23" s="8">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="J23" s="8">
         <v>0</v>
@@ -5939,7 +5939,7 @@
       </c>
       <c r="M23" s="8">
         <f t="shared" si="0"/>
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="N23" s="8">
         <v>0</v>
@@ -5977,7 +5977,7 @@
         <v>14</v>
       </c>
       <c r="I24" s="8">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J24" s="8">
         <v>0</v>
@@ -5990,10 +5990,10 @@
       </c>
       <c r="M24" s="8">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="N24" s="8">
-        <v>411</v>
+        <v>256</v>
       </c>
       <c r="O24" s="8"/>
       <c r="P24" s="8"/>
@@ -6085,17 +6085,17 @@
         <v>0</v>
       </c>
       <c r="K26" s="8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L26" s="8">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="M26" s="8">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
       <c r="N26" s="8">
-        <v>154</v>
+        <v>200</v>
       </c>
       <c r="O26" s="8"/>
       <c r="P26" s="8"/>
@@ -6130,7 +6130,7 @@
         <v>12</v>
       </c>
       <c r="I27" s="8">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J27" s="8">
         <v>0</v>
@@ -6143,10 +6143,10 @@
       </c>
       <c r="M27" s="8">
         <f t="shared" si="0"/>
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N27" s="8">
-        <v>849</v>
+        <v>713</v>
       </c>
       <c r="O27" s="8"/>
       <c r="P27" s="8"/>
@@ -6181,7 +6181,7 @@
         <v>12</v>
       </c>
       <c r="I28" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J28" s="8">
         <v>0</v>
@@ -6194,7 +6194,7 @@
       </c>
       <c r="M28" s="8">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N28" s="8">
         <v>0</v>
@@ -6232,7 +6232,7 @@
         <v>13</v>
       </c>
       <c r="I29" s="8">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="J29" s="8">
         <v>0</v>
@@ -6245,7 +6245,7 @@
       </c>
       <c r="M29" s="8">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="N29" s="8">
         <v>0</v>
@@ -6283,23 +6283,23 @@
         <v>14</v>
       </c>
       <c r="I30" s="8">
+        <v>6</v>
+      </c>
+      <c r="J30" s="8">
+        <v>0</v>
+      </c>
+      <c r="K30" s="8">
+        <v>3</v>
+      </c>
+      <c r="L30" s="8">
         <v>4</v>
-      </c>
-      <c r="J30" s="8">
-        <v>0</v>
-      </c>
-      <c r="K30" s="8">
-        <v>0</v>
-      </c>
-      <c r="L30" s="8">
-        <v>3</v>
       </c>
       <c r="M30" s="8">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="N30" s="8">
-        <v>1307</v>
+        <v>1213</v>
       </c>
       <c r="O30" s="8"/>
       <c r="P30" s="8"/>
@@ -6385,7 +6385,7 @@
         <v>12</v>
       </c>
       <c r="I32" s="8">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J32" s="8">
         <v>0</v>
@@ -6398,10 +6398,10 @@
       </c>
       <c r="M32" s="8">
         <f t="shared" si="0"/>
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="N32" s="8">
-        <v>575</v>
+        <v>517</v>
       </c>
       <c r="O32" s="8"/>
       <c r="P32" s="8"/>
@@ -6436,7 +6436,7 @@
         <v>12</v>
       </c>
       <c r="I33" s="8">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="J33" s="8">
         <v>0</v>
@@ -6445,14 +6445,14 @@
         <v>0</v>
       </c>
       <c r="L33" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M33" s="8">
         <f t="shared" si="0"/>
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="N33" s="8">
-        <v>842</v>
+        <v>733</v>
       </c>
       <c r="O33" s="8"/>
       <c r="P33" s="8"/>
@@ -6487,7 +6487,7 @@
         <v>12</v>
       </c>
       <c r="I34" s="8">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="J34" s="8">
         <v>0</v>
@@ -6500,10 +6500,10 @@
       </c>
       <c r="M34" s="8">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="N34" s="8">
-        <v>899</v>
+        <v>820</v>
       </c>
       <c r="O34" s="8"/>
       <c r="P34" s="8"/>
@@ -6538,7 +6538,7 @@
         <v>12</v>
       </c>
       <c r="I35" s="8">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J35" s="8">
         <v>0</v>
@@ -6551,10 +6551,10 @@
       </c>
       <c r="M35" s="8">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N35" s="8">
-        <v>715</v>
+        <v>703</v>
       </c>
       <c r="O35" s="8"/>
       <c r="P35" s="8"/>
@@ -6605,7 +6605,7 @@
         <v>7</v>
       </c>
       <c r="N36" s="8">
-        <v>616</v>
+        <v>574</v>
       </c>
       <c r="O36" s="8"/>
       <c r="P36" s="8"/>
@@ -6640,7 +6640,7 @@
         <v>13</v>
       </c>
       <c r="I37" s="8">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J37" s="8">
         <v>0</v>
@@ -6653,10 +6653,10 @@
       </c>
       <c r="M37" s="8">
         <f t="shared" si="0"/>
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="N37" s="8">
-        <v>991</v>
+        <v>875</v>
       </c>
       <c r="O37" s="8"/>
       <c r="P37" s="8"/>
@@ -6691,7 +6691,7 @@
         <v>12</v>
       </c>
       <c r="I38" s="8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J38" s="8">
         <v>0</v>
@@ -6704,7 +6704,7 @@
       </c>
       <c r="M38" s="8">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N38" s="8">
         <v>0</v>
@@ -6742,23 +6742,23 @@
         <v>12</v>
       </c>
       <c r="I39" s="8">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J39" s="8">
         <v>0</v>
       </c>
       <c r="K39" s="8">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="L39" s="8">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="M39" s="8">
         <f t="shared" si="0"/>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="N39" s="8">
-        <v>2680</v>
+        <v>2669</v>
       </c>
       <c r="O39" s="8"/>
       <c r="P39" s="8"/>
@@ -6793,7 +6793,7 @@
         <v>12</v>
       </c>
       <c r="I40" s="8">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J40" s="8">
         <v>0</v>
@@ -6806,7 +6806,7 @@
       </c>
       <c r="M40" s="8">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="N40" s="8">
         <v>0</v>
@@ -6844,7 +6844,7 @@
         <v>12</v>
       </c>
       <c r="I41" s="8">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J41" s="8">
         <v>0</v>
@@ -6857,10 +6857,10 @@
       </c>
       <c r="M41" s="8">
         <f t="shared" si="0"/>
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="N41" s="8">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="O41" s="8"/>
       <c r="P41" s="8"/>
@@ -6901,17 +6901,17 @@
         <v>0</v>
       </c>
       <c r="K42" s="8">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L42" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M42" s="8">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
       <c r="N42" s="8">
-        <v>1165</v>
+        <v>979</v>
       </c>
       <c r="O42" s="8"/>
       <c r="P42" s="8"/>
@@ -6946,7 +6946,7 @@
         <v>12</v>
       </c>
       <c r="I43" s="8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J43" s="8">
         <v>0</v>
@@ -6959,7 +6959,7 @@
       </c>
       <c r="M43" s="8">
         <f t="shared" si="0"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N43" s="8">
         <v>0</v>
@@ -6997,7 +6997,7 @@
         <v>12</v>
       </c>
       <c r="I44" s="8">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="J44" s="8">
         <v>0</v>
@@ -7010,10 +7010,10 @@
       </c>
       <c r="M44" s="8">
         <f t="shared" si="0"/>
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="N44" s="8">
-        <v>222</v>
+        <v>165</v>
       </c>
       <c r="O44" s="8"/>
       <c r="P44" s="8"/>
@@ -7064,7 +7064,7 @@
         <v>13</v>
       </c>
       <c r="N45" s="8">
-        <v>600</v>
+        <v>549</v>
       </c>
       <c r="O45" s="8"/>
       <c r="P45" s="8"/>
@@ -7099,7 +7099,7 @@
         <v>12</v>
       </c>
       <c r="I46" s="8">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="J46" s="8">
         <v>0</v>
@@ -7112,10 +7112,10 @@
       </c>
       <c r="M46" s="8">
         <f t="shared" si="0"/>
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="N46" s="8">
-        <v>49</v>
+        <v>0</v>
       </c>
       <c r="O46" s="8"/>
       <c r="P46" s="8"/>
@@ -7166,7 +7166,7 @@
         <v>7</v>
       </c>
       <c r="N47" s="8">
-        <v>755</v>
+        <v>594</v>
       </c>
       <c r="O47" s="8"/>
       <c r="P47" s="8"/>
@@ -7201,7 +7201,7 @@
         <v>12</v>
       </c>
       <c r="I48" s="8">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="J48" s="8">
         <v>0</v>
@@ -7210,14 +7210,14 @@
         <v>0</v>
       </c>
       <c r="L48" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M48" s="8">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="N48" s="8">
-        <v>1500</v>
+        <v>1114</v>
       </c>
       <c r="O48" s="8"/>
       <c r="P48" s="8"/>
@@ -7252,7 +7252,7 @@
         <v>12</v>
       </c>
       <c r="I49" s="8">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J49" s="8">
         <v>0</v>
@@ -7265,10 +7265,10 @@
       </c>
       <c r="M49" s="8">
         <f t="shared" si="0"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="N49" s="8">
-        <v>757</v>
+        <v>603</v>
       </c>
       <c r="O49" s="8"/>
       <c r="P49" s="8"/>
@@ -7319,7 +7319,7 @@
         <v>4</v>
       </c>
       <c r="N50" s="8">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="O50" s="8"/>
       <c r="P50" s="8"/>
@@ -7370,7 +7370,7 @@
         <v>24</v>
       </c>
       <c r="N51" s="8">
-        <v>301</v>
+        <v>263</v>
       </c>
       <c r="O51" s="8"/>
       <c r="P51" s="8"/>
@@ -7405,7 +7405,7 @@
         <v>12</v>
       </c>
       <c r="I52" s="8">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="J52" s="8">
         <v>0</v>
@@ -7418,7 +7418,7 @@
       </c>
       <c r="M52" s="8">
         <f t="shared" si="0"/>
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="N52" s="8">
         <v>0</v>
@@ -7472,7 +7472,7 @@
         <v>9</v>
       </c>
       <c r="N53" s="8">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="O53" s="8"/>
       <c r="P53" s="8"/>
@@ -7523,7 +7523,7 @@
         <v>7</v>
       </c>
       <c r="N54" s="8">
-        <v>433</v>
+        <v>292</v>
       </c>
       <c r="O54" s="8"/>
       <c r="P54" s="8"/>
@@ -7558,7 +7558,7 @@
         <v>12</v>
       </c>
       <c r="I55" s="8">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J55" s="8">
         <v>0</v>
@@ -7571,7 +7571,7 @@
       </c>
       <c r="M55" s="8">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="N55" s="8">
         <v>0</v>
@@ -7618,14 +7618,14 @@
         <v>0</v>
       </c>
       <c r="L56" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M56" s="8">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N56" s="8">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="O56" s="8"/>
       <c r="P56" s="8"/>
@@ -7660,23 +7660,23 @@
         <v>12</v>
       </c>
       <c r="I57" s="8">
-        <v>7</v>
+        <v>19</v>
       </c>
       <c r="J57" s="8">
         <v>0</v>
       </c>
       <c r="K57" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L57" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="M57" s="8">
         <f t="shared" si="0"/>
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="N57" s="8">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="O57" s="8"/>
       <c r="P57" s="8"/>
@@ -7711,23 +7711,23 @@
         <v>12</v>
       </c>
       <c r="I58" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J58" s="8">
         <v>0</v>
       </c>
       <c r="K58" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L58" s="8">
         <v>2</v>
       </c>
       <c r="M58" s="8">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N58" s="8">
-        <v>603</v>
+        <v>587</v>
       </c>
       <c r="O58" s="8"/>
       <c r="P58" s="8"/>
@@ -7813,7 +7813,7 @@
         <v>12</v>
       </c>
       <c r="I60" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J60" s="8">
         <v>0</v>
@@ -7822,14 +7822,14 @@
         <v>0</v>
       </c>
       <c r="L60" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M60" s="8">
         <f t="shared" si="0"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N60" s="8">
-        <v>474</v>
+        <v>354</v>
       </c>
       <c r="O60" s="8"/>
       <c r="P60" s="8"/>
@@ -7864,7 +7864,7 @@
         <v>12</v>
       </c>
       <c r="I61" s="8">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="J61" s="8">
         <v>0</v>
@@ -7877,7 +7877,7 @@
       </c>
       <c r="M61" s="8">
         <f t="shared" si="0"/>
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="N61" s="8">
         <v>0</v>
@@ -7915,7 +7915,7 @@
         <v>12</v>
       </c>
       <c r="I62" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J62" s="8">
         <v>0</v>
@@ -7928,10 +7928,10 @@
       </c>
       <c r="M62" s="8">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N62" s="8">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="O62" s="8"/>
       <c r="P62" s="8"/>
@@ -7966,7 +7966,7 @@
         <v>12</v>
       </c>
       <c r="I63" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J63" s="8">
         <v>0</v>
@@ -7979,10 +7979,10 @@
       </c>
       <c r="M63" s="8">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N63" s="8">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="O63" s="8"/>
       <c r="P63" s="8"/>
@@ -8017,23 +8017,23 @@
         <v>13</v>
       </c>
       <c r="I64" s="8">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="J64" s="8">
         <v>0</v>
       </c>
       <c r="K64" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L64" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M64" s="8">
         <f t="shared" si="0"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="N64" s="8">
-        <v>222</v>
+        <v>411</v>
       </c>
       <c r="O64" s="8"/>
       <c r="P64" s="8"/>
@@ -8068,7 +8068,7 @@
         <v>12</v>
       </c>
       <c r="I65" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J65" s="8">
         <v>0</v>
@@ -8081,10 +8081,10 @@
       </c>
       <c r="M65" s="8">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N65" s="8">
-        <v>848</v>
+        <v>820</v>
       </c>
       <c r="O65" s="8"/>
       <c r="P65" s="8"/>
@@ -8135,7 +8135,7 @@
         <v>4</v>
       </c>
       <c r="N66" s="8">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="O66" s="8"/>
       <c r="P66" s="8"/>
@@ -8186,7 +8186,7 @@
         <v>3</v>
       </c>
       <c r="N67" s="8">
-        <v>664</v>
+        <v>604</v>
       </c>
       <c r="O67" s="8"/>
       <c r="P67" s="8"/>
@@ -8227,17 +8227,17 @@
         <v>0</v>
       </c>
       <c r="K68" s="8">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L68" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M68" s="8">
         <f t="shared" si="1"/>
         <v>7</v>
       </c>
       <c r="N68" s="8">
-        <v>886</v>
+        <v>862</v>
       </c>
       <c r="O68" s="8"/>
       <c r="P68" s="8"/>
@@ -8288,7 +8288,7 @@
         <v>10</v>
       </c>
       <c r="N69" s="8">
-        <v>221</v>
+        <v>132</v>
       </c>
       <c r="O69" s="8"/>
       <c r="P69" s="8"/>
@@ -8323,7 +8323,7 @@
         <v>16</v>
       </c>
       <c r="I70" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J70" s="8">
         <v>0</v>
@@ -8336,7 +8336,7 @@
       </c>
       <c r="M70" s="8">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N70" s="8">
         <v>543</v>
@@ -8374,7 +8374,7 @@
         <v>12</v>
       </c>
       <c r="I71" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J71" s="8">
         <v>0</v>
@@ -8387,7 +8387,7 @@
       </c>
       <c r="M71" s="8">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N71" s="8">
         <v>0</v>
@@ -8425,7 +8425,7 @@
         <v>12</v>
       </c>
       <c r="I72" s="8">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J72" s="8">
         <v>0</v>
@@ -8438,10 +8438,10 @@
       </c>
       <c r="M72" s="8">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N72" s="8">
-        <v>528</v>
+        <v>470</v>
       </c>
       <c r="O72" s="8"/>
       <c r="P72" s="8"/>
@@ -8482,14 +8482,14 @@
         <v>0</v>
       </c>
       <c r="K73" s="8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L73" s="8">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="M73" s="8">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="N73" s="8">
         <v>169</v>
@@ -8543,7 +8543,7 @@
         <v>6</v>
       </c>
       <c r="N74" s="8">
-        <v>138</v>
+        <v>118</v>
       </c>
       <c r="O74" s="8"/>
       <c r="P74" s="8"/>
@@ -8629,7 +8629,7 @@
         <v>13</v>
       </c>
       <c r="I76" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J76" s="8">
         <v>0</v>
@@ -8642,10 +8642,10 @@
       </c>
       <c r="M76" s="8">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N76" s="8">
-        <v>871</v>
+        <v>874</v>
       </c>
       <c r="O76" s="8"/>
       <c r="P76" s="8"/>
@@ -8696,7 +8696,7 @@
         <v>5</v>
       </c>
       <c r="N77" s="8">
-        <v>509</v>
+        <v>387</v>
       </c>
       <c r="O77" s="8"/>
       <c r="P77" s="8"/>
@@ -8731,23 +8731,23 @@
         <v>12</v>
       </c>
       <c r="I78" s="8">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="J78" s="8">
         <v>0</v>
       </c>
       <c r="K78" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L78" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M78" s="8">
         <f t="shared" si="1"/>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N78" s="8">
-        <v>300</v>
+        <v>221</v>
       </c>
       <c r="O78" s="8"/>
       <c r="P78" s="8"/>
@@ -8849,7 +8849,7 @@
         <v>3</v>
       </c>
       <c r="N80" s="8">
-        <v>346</v>
+        <v>239</v>
       </c>
       <c r="O80" s="8"/>
       <c r="P80" s="8"/>
@@ -8951,7 +8951,7 @@
         <v>5</v>
       </c>
       <c r="N82" s="8">
-        <v>222</v>
+        <v>172</v>
       </c>
       <c r="O82" s="8"/>
       <c r="P82" s="8"/>
@@ -9002,7 +9002,7 @@
         <v>4</v>
       </c>
       <c r="N83" s="8">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="O83" s="8"/>
       <c r="P83" s="8"/>
@@ -9088,7 +9088,7 @@
         <v>14</v>
       </c>
       <c r="I85" s="8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J85" s="8">
         <v>0</v>
@@ -9101,10 +9101,10 @@
       </c>
       <c r="M85" s="8">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N85" s="8">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="O85" s="8"/>
       <c r="P85" s="8"/>
@@ -9139,7 +9139,7 @@
         <v>12</v>
       </c>
       <c r="I86" s="8">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J86" s="8">
         <v>0</v>
@@ -9152,10 +9152,10 @@
       </c>
       <c r="M86" s="8">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N86" s="8">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O86" s="8"/>
       <c r="P86" s="8"/>
@@ -9241,7 +9241,7 @@
         <v>12</v>
       </c>
       <c r="I88" s="8">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="J88" s="8">
         <v>0</v>
@@ -9254,10 +9254,10 @@
       </c>
       <c r="M88" s="8">
         <f t="shared" si="1"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="N88" s="8">
-        <v>258</v>
+        <v>155</v>
       </c>
       <c r="O88" s="8"/>
       <c r="P88" s="8"/>
@@ -9292,7 +9292,7 @@
         <v>12</v>
       </c>
       <c r="I89" s="8">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J89" s="8">
         <v>0</v>
@@ -9305,10 +9305,10 @@
       </c>
       <c r="M89" s="8">
         <f t="shared" si="1"/>
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="N89" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O89" s="8"/>
       <c r="P89" s="8"/>
@@ -9359,7 +9359,7 @@
         <v>5</v>
       </c>
       <c r="N90" s="8">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="O90" s="8"/>
       <c r="P90" s="8"/>
@@ -9400,17 +9400,17 @@
         <v>0</v>
       </c>
       <c r="K91" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L91" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M91" s="8">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="N91" s="8">
-        <v>938</v>
+        <v>864</v>
       </c>
       <c r="O91" s="8"/>
       <c r="P91" s="8"/>
@@ -9454,14 +9454,14 @@
         <v>0</v>
       </c>
       <c r="L92" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M92" s="8">
         <f t="shared" si="1"/>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N92" s="8">
-        <v>40</v>
+        <v>0</v>
       </c>
       <c r="O92" s="8"/>
       <c r="P92" s="8"/>
@@ -9614,7 +9614,7 @@
         <v>6</v>
       </c>
       <c r="N95" s="8">
-        <v>139</v>
+        <v>128</v>
       </c>
       <c r="O95" s="8"/>
       <c r="P95" s="8"/>
@@ -9649,7 +9649,7 @@
         <v>13</v>
       </c>
       <c r="I96" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J96" s="8">
         <v>0</v>
@@ -9662,10 +9662,10 @@
       </c>
       <c r="M96" s="8">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N96" s="8">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="O96" s="8"/>
       <c r="P96" s="8"/>
@@ -9700,23 +9700,23 @@
         <v>14</v>
       </c>
       <c r="I97" s="8">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J97" s="8">
         <v>0</v>
       </c>
       <c r="K97" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L97" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M97" s="8">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="N97" s="8">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="O97" s="8"/>
       <c r="P97" s="8"/>
@@ -9904,23 +9904,23 @@
         <v>15</v>
       </c>
       <c r="I101" s="8">
+        <v>2</v>
+      </c>
+      <c r="J101" s="8">
+        <v>0</v>
+      </c>
+      <c r="K101" s="8">
+        <v>0</v>
+      </c>
+      <c r="L101" s="8">
         <v>1</v>
-      </c>
-      <c r="J101" s="8">
-        <v>0</v>
-      </c>
-      <c r="K101" s="8">
-        <v>0</v>
-      </c>
-      <c r="L101" s="8">
-        <v>0</v>
       </c>
       <c r="M101" s="8">
         <f t="shared" si="1"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N101" s="8">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="O101" s="8"/>
       <c r="P101" s="8"/>
@@ -9955,23 +9955,23 @@
         <v>14</v>
       </c>
       <c r="I102" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J102" s="8">
         <v>0</v>
       </c>
       <c r="K102" s="8">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L102" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M102" s="8">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N102" s="8">
-        <v>385</v>
+        <v>369</v>
       </c>
       <c r="O102" s="8"/>
       <c r="P102" s="8"/>
@@ -10022,7 +10022,7 @@
         <v>5</v>
       </c>
       <c r="N103" s="8">
-        <v>0</v>
+        <v>284</v>
       </c>
       <c r="O103" s="8"/>
       <c r="P103" s="8"/>
@@ -10108,7 +10108,7 @@
         <v>12</v>
       </c>
       <c r="I105" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J105" s="8">
         <v>0</v>
@@ -10121,10 +10121,10 @@
       </c>
       <c r="M105" s="8">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N105" s="8">
-        <v>372</v>
+        <v>365</v>
       </c>
       <c r="O105" s="8"/>
       <c r="P105" s="8"/>
@@ -10328,7 +10328,7 @@
         <v>4</v>
       </c>
       <c r="N109" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O109" s="8"/>
       <c r="P109" s="8"/>
@@ -10363,7 +10363,7 @@
         <v>13</v>
       </c>
       <c r="I110" s="8">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="J110" s="8">
         <v>0</v>
@@ -10376,10 +10376,10 @@
       </c>
       <c r="M110" s="8">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N110" s="8">
-        <v>520</v>
+        <v>540</v>
       </c>
       <c r="O110" s="8"/>
       <c r="P110" s="8"/>
@@ -10465,7 +10465,7 @@
         <v>12</v>
       </c>
       <c r="I112" s="8">
-        <v>240</v>
+        <v>224</v>
       </c>
       <c r="J112" s="8">
         <v>0</v>
@@ -10478,10 +10478,10 @@
       </c>
       <c r="M112" s="8">
         <f t="shared" si="1"/>
-        <v>240</v>
+        <v>224</v>
       </c>
       <c r="N112" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O112" s="8"/>
       <c r="P112" s="8"/>
@@ -10525,14 +10525,14 @@
         <v>0</v>
       </c>
       <c r="L113" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M113" s="8">
         <f t="shared" si="1"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="N113" s="8">
-        <v>733</v>
+        <v>653</v>
       </c>
       <c r="O113" s="8"/>
       <c r="P113" s="8"/>
@@ -10583,7 +10583,7 @@
         <v>6</v>
       </c>
       <c r="N114" s="8">
-        <v>531</v>
+        <v>357</v>
       </c>
       <c r="O114" s="8"/>
       <c r="P114" s="8"/>
@@ -10634,7 +10634,7 @@
         <v>9</v>
       </c>
       <c r="N115" s="8">
-        <v>507</v>
+        <v>484</v>
       </c>
       <c r="O115" s="8"/>
       <c r="P115" s="8"/>
@@ -10669,7 +10669,7 @@
         <v>12</v>
       </c>
       <c r="I116" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J116" s="8">
         <v>0</v>
@@ -10682,10 +10682,10 @@
       </c>
       <c r="M116" s="8">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N116" s="8">
-        <v>633</v>
+        <v>534</v>
       </c>
       <c r="O116" s="8"/>
       <c r="P116" s="8"/>
@@ -10720,23 +10720,23 @@
         <v>12</v>
       </c>
       <c r="I117" s="8">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="J117" s="8">
         <v>0</v>
       </c>
       <c r="K117" s="8">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L117" s="8">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="M117" s="8">
         <f t="shared" si="1"/>
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="N117" s="8">
-        <v>111</v>
+        <v>10</v>
       </c>
       <c r="O117" s="8"/>
       <c r="P117" s="8"/>
@@ -10787,7 +10787,7 @@
         <v>6</v>
       </c>
       <c r="N118" s="8">
-        <v>162</v>
+        <v>150</v>
       </c>
       <c r="O118" s="8"/>
       <c r="P118" s="8"/>
@@ -10838,7 +10838,7 @@
         <v>8</v>
       </c>
       <c r="N119" s="8">
-        <v>461</v>
+        <v>435</v>
       </c>
       <c r="O119" s="8"/>
       <c r="P119" s="8"/>
@@ -10873,7 +10873,7 @@
         <v>14</v>
       </c>
       <c r="I120" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J120" s="8">
         <v>0</v>
@@ -10886,10 +10886,10 @@
       </c>
       <c r="M120" s="8">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N120" s="8">
-        <v>41</v>
+        <v>1</v>
       </c>
       <c r="O120" s="8"/>
       <c r="P120" s="8"/>
@@ -10991,7 +10991,7 @@
         <v>2</v>
       </c>
       <c r="N122" s="8">
-        <v>950</v>
+        <v>889</v>
       </c>
       <c r="O122" s="8"/>
       <c r="P122" s="8"/>
@@ -11144,7 +11144,7 @@
         <v>6</v>
       </c>
       <c r="N125" s="8">
-        <v>81</v>
+        <v>4</v>
       </c>
       <c r="O125" s="8"/>
       <c r="P125" s="8"/>
@@ -11297,7 +11297,7 @@
         <v>3</v>
       </c>
       <c r="N128" s="8">
-        <v>804</v>
+        <v>795</v>
       </c>
       <c r="O128" s="8"/>
       <c r="P128" s="8"/>
@@ -11383,23 +11383,23 @@
         <v>12</v>
       </c>
       <c r="I130" s="8">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J130" s="8">
         <v>0</v>
       </c>
       <c r="K130" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L130" s="8">
         <v>1</v>
       </c>
       <c r="M130" s="8">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N130" s="8">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="O130" s="8"/>
       <c r="P130" s="8"/>
@@ -11434,7 +11434,7 @@
         <v>14</v>
       </c>
       <c r="I131" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J131" s="8">
         <v>0</v>
@@ -11447,10 +11447,10 @@
       </c>
       <c r="M131" s="8">
         <f t="shared" ref="M131:M194" si="2">I131+J131+K131+L131</f>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N131" s="8">
-        <v>463</v>
+        <v>438</v>
       </c>
       <c r="O131" s="8"/>
       <c r="P131" s="8"/>
@@ -11485,7 +11485,7 @@
         <v>12</v>
       </c>
       <c r="I132" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J132" s="8">
         <v>0</v>
@@ -11498,10 +11498,10 @@
       </c>
       <c r="M132" s="8">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N132" s="8">
-        <v>834</v>
+        <v>828</v>
       </c>
       <c r="O132" s="8"/>
       <c r="P132" s="8"/>
@@ -11536,23 +11536,23 @@
         <v>12</v>
       </c>
       <c r="I133" s="8">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J133" s="8">
         <v>0</v>
       </c>
       <c r="K133" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L133" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M133" s="8">
         <f t="shared" si="2"/>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="N133" s="8">
-        <v>295</v>
+        <v>8</v>
       </c>
       <c r="O133" s="8"/>
       <c r="P133" s="8"/>
@@ -11603,7 +11603,7 @@
         <v>4</v>
       </c>
       <c r="N134" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O134" s="8"/>
       <c r="P134" s="8"/>
@@ -11638,23 +11638,23 @@
         <v>15</v>
       </c>
       <c r="I135" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J135" s="8">
         <v>0</v>
       </c>
       <c r="K135" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L135" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M135" s="8">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N135" s="8">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="O135" s="8"/>
       <c r="P135" s="8"/>
@@ -11695,17 +11695,17 @@
         <v>0</v>
       </c>
       <c r="K136" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L136" s="8">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M136" s="8">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="N136" s="8">
-        <v>350</v>
+        <v>292</v>
       </c>
       <c r="O136" s="8"/>
       <c r="P136" s="8"/>
@@ -11740,7 +11740,7 @@
         <v>15</v>
       </c>
       <c r="I137" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J137" s="8">
         <v>0</v>
@@ -11753,10 +11753,10 @@
       </c>
       <c r="M137" s="8">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N137" s="8">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="O137" s="8"/>
       <c r="P137" s="8"/>
@@ -11791,23 +11791,23 @@
         <v>12</v>
       </c>
       <c r="I138" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J138" s="8">
         <v>0</v>
       </c>
       <c r="K138" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L138" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M138" s="8">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N138" s="8">
-        <v>964</v>
+        <v>969</v>
       </c>
       <c r="O138" s="8"/>
       <c r="P138" s="8"/>
@@ -11851,14 +11851,14 @@
         <v>0</v>
       </c>
       <c r="L139" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M139" s="8">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N139" s="8">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="O139" s="8"/>
       <c r="P139" s="8"/>
@@ -11893,7 +11893,7 @@
         <v>15</v>
       </c>
       <c r="I140" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J140" s="8">
         <v>0</v>
@@ -11906,10 +11906,10 @@
       </c>
       <c r="M140" s="8">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N140" s="8">
-        <v>447</v>
+        <v>445</v>
       </c>
       <c r="O140" s="8"/>
       <c r="P140" s="8"/>
@@ -11953,11 +11953,11 @@
         <v>0</v>
       </c>
       <c r="L141" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M141" s="8">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N141" s="8">
         <v>0</v>
@@ -12055,11 +12055,11 @@
         <v>0</v>
       </c>
       <c r="L143" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M143" s="8">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N143" s="8">
         <v>0</v>
@@ -12164,7 +12164,7 @@
         <v>4</v>
       </c>
       <c r="N145" s="8">
-        <v>823</v>
+        <v>778</v>
       </c>
       <c r="O145" s="8"/>
       <c r="P145" s="8"/>
@@ -12199,7 +12199,7 @@
         <v>16</v>
       </c>
       <c r="I146" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J146" s="8">
         <v>0</v>
@@ -12212,7 +12212,7 @@
       </c>
       <c r="M146" s="8">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N146" s="8">
         <v>0</v>
@@ -12250,7 +12250,7 @@
         <v>14</v>
       </c>
       <c r="I147" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J147" s="8">
         <v>0</v>
@@ -12263,10 +12263,10 @@
       </c>
       <c r="M147" s="8">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N147" s="8">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="O147" s="8"/>
       <c r="P147" s="8"/>
@@ -12317,7 +12317,7 @@
         <v>2</v>
       </c>
       <c r="N148" s="8">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="O148" s="8"/>
       <c r="P148" s="8"/>
@@ -12361,14 +12361,14 @@
         <v>0</v>
       </c>
       <c r="L149" s="8">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M149" s="8">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="N149" s="8">
-        <v>173</v>
+        <v>139</v>
       </c>
       <c r="O149" s="8"/>
       <c r="P149" s="8"/>
@@ -12409,17 +12409,17 @@
         <v>0</v>
       </c>
       <c r="K150" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L150" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M150" s="8">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
       <c r="N150" s="8">
-        <v>566</v>
+        <v>552</v>
       </c>
       <c r="O150" s="8"/>
       <c r="P150" s="8"/>
@@ -12470,7 +12470,7 @@
         <v>3</v>
       </c>
       <c r="N151" s="8">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O151" s="8"/>
       <c r="P151" s="8"/>
@@ -12521,7 +12521,7 @@
         <v>3</v>
       </c>
       <c r="N152" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O152" s="8"/>
       <c r="P152" s="8"/>
@@ -12565,11 +12565,11 @@
         <v>0</v>
       </c>
       <c r="L153" s="8">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M153" s="8">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="N153" s="8">
         <v>0</v>
@@ -12623,7 +12623,7 @@
         <v>2</v>
       </c>
       <c r="N154" s="8">
-        <v>0</v>
+        <v>454</v>
       </c>
       <c r="O154" s="8"/>
       <c r="P154" s="8"/>
@@ -12929,7 +12929,7 @@
         <v>3</v>
       </c>
       <c r="N160" s="8">
-        <v>0</v>
+        <v>445</v>
       </c>
       <c r="O160" s="8"/>
       <c r="P160" s="8"/>
@@ -12980,7 +12980,7 @@
         <v>5</v>
       </c>
       <c r="N161" s="8">
-        <v>398</v>
+        <v>386</v>
       </c>
       <c r="O161" s="8"/>
       <c r="P161" s="8"/>
@@ -13015,7 +13015,7 @@
         <v>13</v>
       </c>
       <c r="I162" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J162" s="8">
         <v>0</v>
@@ -13028,10 +13028,10 @@
       </c>
       <c r="M162" s="8">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N162" s="8">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="O162" s="8"/>
       <c r="P162" s="8"/>
@@ -13082,7 +13082,7 @@
         <v>4</v>
       </c>
       <c r="N163" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O163" s="8"/>
       <c r="P163" s="8"/>
@@ -13133,7 +13133,7 @@
         <v>2</v>
       </c>
       <c r="N164" s="8">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="O164" s="8"/>
       <c r="P164" s="8"/>
@@ -13184,7 +13184,7 @@
         <v>9</v>
       </c>
       <c r="N165" s="8">
-        <v>1152</v>
+        <v>1070</v>
       </c>
       <c r="O165" s="8"/>
       <c r="P165" s="8"/>
@@ -13235,7 +13235,7 @@
         <v>2</v>
       </c>
       <c r="N166" s="8">
-        <v>883</v>
+        <v>0</v>
       </c>
       <c r="O166" s="8"/>
       <c r="P166" s="8"/>
@@ -13321,23 +13321,23 @@
         <v>14</v>
       </c>
       <c r="I168" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J168" s="8">
         <v>0</v>
       </c>
       <c r="K168" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L168" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M168" s="8">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N168" s="8">
-        <v>173</v>
+        <v>124</v>
       </c>
       <c r="O168" s="8"/>
       <c r="P168" s="8"/>
@@ -13439,7 +13439,7 @@
         <v>1</v>
       </c>
       <c r="N170" s="8">
-        <v>652</v>
+        <v>640</v>
       </c>
       <c r="O170" s="8"/>
       <c r="P170" s="8"/>
@@ -13541,7 +13541,7 @@
         <v>1</v>
       </c>
       <c r="N172" s="8">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="O172" s="8"/>
       <c r="P172" s="8"/>
@@ -13585,14 +13585,14 @@
         <v>0</v>
       </c>
       <c r="L173" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M173" s="8">
         <f t="shared" si="2"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N173" s="8">
-        <v>552</v>
+        <v>529</v>
       </c>
       <c r="O173" s="8"/>
       <c r="P173" s="8"/>
@@ -13898,7 +13898,7 @@
         <v>2</v>
       </c>
       <c r="N179" s="8">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="O179" s="8"/>
       <c r="P179" s="8"/>
@@ -13933,23 +13933,23 @@
         <v>13</v>
       </c>
       <c r="I180" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J180" s="8">
         <v>0</v>
       </c>
       <c r="K180" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L180" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M180" s="8">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N180" s="8">
-        <v>451</v>
+        <v>379</v>
       </c>
       <c r="O180" s="8"/>
       <c r="P180" s="8"/>
@@ -14000,7 +14000,7 @@
         <v>3</v>
       </c>
       <c r="N181" s="8">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="O181" s="8"/>
       <c r="P181" s="8"/>
@@ -14086,7 +14086,7 @@
         <v>12</v>
       </c>
       <c r="I183" s="8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J183" s="8">
         <v>0</v>
@@ -14099,10 +14099,10 @@
       </c>
       <c r="M183" s="8">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N183" s="8">
-        <v>420</v>
+        <v>377</v>
       </c>
       <c r="O183" s="8"/>
       <c r="P183" s="8"/>
@@ -14188,7 +14188,7 @@
         <v>12</v>
       </c>
       <c r="I185" s="8">
-        <v>460</v>
+        <v>379</v>
       </c>
       <c r="J185" s="8">
         <v>0</v>
@@ -14201,7 +14201,7 @@
       </c>
       <c r="M185" s="8">
         <f t="shared" si="2"/>
-        <v>460</v>
+        <v>379</v>
       </c>
       <c r="N185" s="8">
         <v>1659</v>
@@ -14255,7 +14255,7 @@
         <v>6</v>
       </c>
       <c r="N186" s="8">
-        <v>791</v>
+        <v>678</v>
       </c>
       <c r="O186" s="8"/>
       <c r="P186" s="8"/>
@@ -14306,7 +14306,7 @@
         <v>1</v>
       </c>
       <c r="N187" s="8">
-        <v>134</v>
+        <v>89</v>
       </c>
       <c r="O187" s="8"/>
       <c r="P187" s="8"/>
@@ -14341,7 +14341,7 @@
         <v>15</v>
       </c>
       <c r="I188" s="8">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J188" s="8">
         <v>0</v>
@@ -14354,10 +14354,10 @@
       </c>
       <c r="M188" s="8">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N188" s="8">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="O188" s="8"/>
       <c r="P188" s="8"/>
@@ -14443,7 +14443,7 @@
         <v>12</v>
       </c>
       <c r="I190" s="8">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J190" s="8">
         <v>0</v>
@@ -14456,10 +14456,10 @@
       </c>
       <c r="M190" s="8">
         <f t="shared" si="2"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N190" s="8">
-        <v>307</v>
+        <v>290</v>
       </c>
       <c r="O190" s="8"/>
       <c r="P190" s="8"/>
@@ -14494,7 +14494,7 @@
         <v>12</v>
       </c>
       <c r="I191" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J191" s="8">
         <v>0</v>
@@ -14507,10 +14507,10 @@
       </c>
       <c r="M191" s="8">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N191" s="8">
-        <v>671</v>
+        <v>525</v>
       </c>
       <c r="O191" s="8"/>
       <c r="P191" s="8"/>
@@ -14612,7 +14612,7 @@
         <v>3</v>
       </c>
       <c r="N193" s="8">
-        <v>512</v>
+        <v>516</v>
       </c>
       <c r="O193" s="8"/>
       <c r="P193" s="8"/>
@@ -14647,7 +14647,7 @@
         <v>15</v>
       </c>
       <c r="I194" s="8">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J194" s="8">
         <v>0</v>
@@ -14656,14 +14656,14 @@
         <v>0</v>
       </c>
       <c r="L194" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M194" s="8">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="N194" s="8">
-        <v>250</v>
+        <v>264</v>
       </c>
       <c r="O194" s="8"/>
       <c r="P194" s="8"/>
@@ -14806,17 +14806,17 @@
         <v>0</v>
       </c>
       <c r="K197" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L197" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M197" s="8">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
       <c r="N197" s="8">
-        <v>439</v>
+        <v>323</v>
       </c>
       <c r="O197" s="8"/>
       <c r="P197" s="8"/>
@@ -15122,7 +15122,7 @@
         <v>2</v>
       </c>
       <c r="N203" s="8">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="O203" s="8"/>
       <c r="P203" s="8"/>
@@ -15326,7 +15326,7 @@
         <v>4</v>
       </c>
       <c r="N207" s="8">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="O207" s="8"/>
       <c r="P207" s="8"/>
@@ -15361,23 +15361,23 @@
         <v>14</v>
       </c>
       <c r="I208" s="8">
+        <v>1</v>
+      </c>
+      <c r="J208" s="8">
+        <v>0</v>
+      </c>
+      <c r="K208" s="8">
         <v>2</v>
       </c>
-      <c r="J208" s="8">
-        <v>0</v>
-      </c>
-      <c r="K208" s="8">
-        <v>0</v>
-      </c>
       <c r="L208" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M208" s="8">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N208" s="8">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="O208" s="8"/>
       <c r="P208" s="8"/>
@@ -15530,7 +15530,7 @@
         <v>3</v>
       </c>
       <c r="N211" s="8">
-        <v>709</v>
+        <v>703</v>
       </c>
       <c r="O211" s="8"/>
       <c r="P211" s="8"/>
@@ -15565,7 +15565,7 @@
         <v>14</v>
       </c>
       <c r="I212" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J212" s="8">
         <v>0</v>
@@ -15578,7 +15578,7 @@
       </c>
       <c r="M212" s="8">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N212" s="8">
         <v>0</v>
@@ -15667,23 +15667,23 @@
         <v>14</v>
       </c>
       <c r="I214" s="8">
+        <v>2</v>
+      </c>
+      <c r="J214" s="8">
+        <v>0</v>
+      </c>
+      <c r="K214" s="8">
+        <v>0</v>
+      </c>
+      <c r="L214" s="8">
         <v>1</v>
-      </c>
-      <c r="J214" s="8">
-        <v>0</v>
-      </c>
-      <c r="K214" s="8">
-        <v>0</v>
-      </c>
-      <c r="L214" s="8">
-        <v>0</v>
       </c>
       <c r="M214" s="8">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N214" s="8">
-        <v>454</v>
+        <v>435</v>
       </c>
       <c r="O214" s="8"/>
       <c r="P214" s="8"/>
@@ -15718,7 +15718,7 @@
         <v>14</v>
       </c>
       <c r="I215" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J215" s="8">
         <v>0</v>
@@ -15731,10 +15731,10 @@
       </c>
       <c r="M215" s="8">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N215" s="8">
-        <v>638</v>
+        <v>614</v>
       </c>
       <c r="O215" s="8"/>
       <c r="P215" s="8"/>
@@ -15836,7 +15836,7 @@
         <v>3</v>
       </c>
       <c r="N217" s="8">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="O217" s="8"/>
       <c r="P217" s="8"/>
@@ -15887,7 +15887,7 @@
         <v>4</v>
       </c>
       <c r="N218" s="8">
-        <v>0</v>
+        <v>191</v>
       </c>
       <c r="O218" s="8"/>
       <c r="P218" s="8"/>
@@ -15938,7 +15938,7 @@
         <v>4</v>
       </c>
       <c r="N219" s="8">
-        <v>0</v>
+        <v>256</v>
       </c>
       <c r="O219" s="8"/>
       <c r="P219" s="8"/>
@@ -16040,7 +16040,7 @@
         <v>2</v>
       </c>
       <c r="N221" s="8">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O221" s="8"/>
       <c r="P221" s="8"/>
@@ -16126,20 +16126,20 @@
         <v>15</v>
       </c>
       <c r="I223" s="8">
+        <v>1</v>
+      </c>
+      <c r="J223" s="8">
+        <v>0</v>
+      </c>
+      <c r="K223" s="8">
         <v>2</v>
       </c>
-      <c r="J223" s="8">
-        <v>0</v>
-      </c>
-      <c r="K223" s="8">
-        <v>0</v>
-      </c>
       <c r="L223" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M223" s="8">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N223" s="8">
         <v>0</v>
@@ -16177,20 +16177,20 @@
         <v>13</v>
       </c>
       <c r="I224" s="8">
+        <v>2</v>
+      </c>
+      <c r="J224" s="8">
+        <v>0</v>
+      </c>
+      <c r="K224" s="8">
         <v>1</v>
       </c>
-      <c r="J224" s="8">
-        <v>0</v>
-      </c>
-      <c r="K224" s="8">
-        <v>0</v>
-      </c>
       <c r="L224" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M224" s="8">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N224" s="8">
         <v>174</v>
@@ -16244,7 +16244,7 @@
         <v>3</v>
       </c>
       <c r="N225" s="8">
-        <v>467</v>
+        <v>422</v>
       </c>
       <c r="O225" s="8"/>
       <c r="P225" s="8"/>
@@ -16295,7 +16295,7 @@
         <v>0</v>
       </c>
       <c r="N226" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O226" s="8"/>
       <c r="P226" s="8"/>
@@ -16397,7 +16397,7 @@
         <v>2</v>
       </c>
       <c r="N228" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O228" s="8"/>
       <c r="P228" s="8"/>
@@ -16432,7 +16432,7 @@
         <v>15</v>
       </c>
       <c r="I229" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J229" s="8">
         <v>0</v>
@@ -16445,10 +16445,10 @@
       </c>
       <c r="M229" s="8">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N229" s="8">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="O229" s="8"/>
       <c r="P229" s="8"/>
@@ -16489,10 +16489,10 @@
         <v>0</v>
       </c>
       <c r="K230" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L230" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M230" s="8">
         <f t="shared" si="3"/>
@@ -16585,7 +16585,7 @@
         <v>12</v>
       </c>
       <c r="I232" s="8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="J232" s="8">
         <v>0</v>
@@ -16598,10 +16598,10 @@
       </c>
       <c r="M232" s="8">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N232" s="8">
-        <v>383</v>
+        <v>316</v>
       </c>
       <c r="O232" s="8"/>
       <c r="P232" s="8"/>
@@ -16636,23 +16636,23 @@
         <v>15</v>
       </c>
       <c r="I233" s="8">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J233" s="8">
         <v>0</v>
       </c>
       <c r="K233" s="8">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L233" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M233" s="8">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N233" s="8">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="O233" s="8"/>
       <c r="P233" s="8"/>
@@ -16687,7 +16687,7 @@
         <v>15</v>
       </c>
       <c r="I234" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J234" s="8">
         <v>0</v>
@@ -16700,10 +16700,10 @@
       </c>
       <c r="M234" s="8">
         <f t="shared" si="3"/>
+        <v>1</v>
+      </c>
+      <c r="N234" s="8">
         <v>2</v>
-      </c>
-      <c r="N234" s="8">
-        <v>0</v>
       </c>
       <c r="O234" s="8"/>
       <c r="P234" s="8"/>
@@ -16754,7 +16754,7 @@
         <v>2</v>
       </c>
       <c r="N235" s="8">
-        <v>182</v>
+        <v>37</v>
       </c>
       <c r="O235" s="8"/>
       <c r="P235" s="8"/>
@@ -16846,17 +16846,17 @@
         <v>0</v>
       </c>
       <c r="K237" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L237" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M237" s="8">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
       <c r="N237" s="8">
-        <v>775</v>
+        <v>767</v>
       </c>
       <c r="O237" s="8"/>
       <c r="P237" s="8"/>
@@ -16907,7 +16907,7 @@
         <v>4</v>
       </c>
       <c r="N238" s="8">
-        <v>430</v>
+        <v>413</v>
       </c>
       <c r="O238" s="8"/>
       <c r="P238" s="8"/>
@@ -16958,7 +16958,7 @@
         <v>3</v>
       </c>
       <c r="N239" s="8">
-        <v>119</v>
+        <v>102</v>
       </c>
       <c r="O239" s="8"/>
       <c r="P239" s="8"/>
@@ -16999,17 +16999,17 @@
         <v>0</v>
       </c>
       <c r="K240" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L240" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M240" s="8">
         <f t="shared" si="3"/>
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="N240" s="8">
-        <v>295</v>
+        <v>242</v>
       </c>
       <c r="O240" s="8"/>
       <c r="P240" s="8"/>
@@ -17060,7 +17060,7 @@
         <v>3</v>
       </c>
       <c r="N241" s="8">
-        <v>248</v>
+        <v>215</v>
       </c>
       <c r="O241" s="8"/>
       <c r="P241" s="8"/>
@@ -17095,7 +17095,7 @@
         <v>12</v>
       </c>
       <c r="I242" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J242" s="8">
         <v>0</v>
@@ -17108,10 +17108,10 @@
       </c>
       <c r="M242" s="8">
         <f t="shared" si="3"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N242" s="8">
-        <v>667</v>
+        <v>663</v>
       </c>
       <c r="O242" s="8"/>
       <c r="P242" s="8"/>
@@ -17146,23 +17146,23 @@
         <v>15</v>
       </c>
       <c r="I243" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J243" s="8">
         <v>0</v>
       </c>
       <c r="K243" s="8">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L243" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M243" s="8">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N243" s="8">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="O243" s="8"/>
       <c r="P243" s="8"/>
@@ -17315,7 +17315,7 @@
         <v>3</v>
       </c>
       <c r="N246" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O246" s="8"/>
       <c r="P246" s="8"/>
@@ -17350,7 +17350,7 @@
         <v>13</v>
       </c>
       <c r="I247" s="8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J247" s="8">
         <v>0</v>
@@ -17363,10 +17363,10 @@
       </c>
       <c r="M247" s="8">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N247" s="8">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="O247" s="8"/>
       <c r="P247" s="8"/>
@@ -17452,7 +17452,7 @@
         <v>13</v>
       </c>
       <c r="I249" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J249" s="8">
         <v>0</v>
@@ -17465,7 +17465,7 @@
       </c>
       <c r="M249" s="8">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N249" s="8">
         <v>0</v>
@@ -17503,7 +17503,7 @@
         <v>12</v>
       </c>
       <c r="I250" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J250" s="8">
         <v>0</v>
@@ -17516,10 +17516,10 @@
       </c>
       <c r="M250" s="8">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N250" s="8">
-        <v>1383</v>
+        <v>1374</v>
       </c>
       <c r="O250" s="8"/>
       <c r="P250" s="8"/>
@@ -17570,7 +17570,7 @@
         <v>2</v>
       </c>
       <c r="N251" s="8">
-        <v>1212</v>
+        <v>1199</v>
       </c>
       <c r="O251" s="8"/>
       <c r="P251" s="8"/>
@@ -17656,7 +17656,7 @@
         <v>14</v>
       </c>
       <c r="I253" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J253" s="8">
         <v>0</v>
@@ -17669,7 +17669,7 @@
       </c>
       <c r="M253" s="8">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N253" s="8">
         <v>1196</v>
@@ -17707,7 +17707,7 @@
         <v>14</v>
       </c>
       <c r="I254" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J254" s="8">
         <v>0</v>
@@ -17720,7 +17720,7 @@
       </c>
       <c r="M254" s="8">
         <f t="shared" si="3"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N254" s="8">
         <v>519</v>
@@ -17774,7 +17774,7 @@
         <v>3</v>
       </c>
       <c r="N255" s="8">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="O255" s="8"/>
       <c r="P255" s="8"/>
@@ -17825,7 +17825,7 @@
         <v>3</v>
       </c>
       <c r="N256" s="8">
-        <v>1030</v>
+        <v>1023</v>
       </c>
       <c r="O256" s="8"/>
       <c r="P256" s="8"/>
@@ -17876,7 +17876,7 @@
         <v>4</v>
       </c>
       <c r="N257" s="8">
-        <v>331</v>
+        <v>311</v>
       </c>
       <c r="O257" s="8"/>
       <c r="P257" s="8"/>
@@ -17911,7 +17911,7 @@
         <v>16</v>
       </c>
       <c r="I258" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J258" s="8">
         <v>0</v>
@@ -17924,10 +17924,10 @@
       </c>
       <c r="M258" s="8">
         <f t="shared" si="3"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N258" s="8">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="O258" s="8"/>
       <c r="P258" s="8"/>
@@ -17978,7 +17978,7 @@
         <v>3</v>
       </c>
       <c r="N259" s="8">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="O259" s="8"/>
       <c r="P259" s="8"/>
@@ -18013,23 +18013,23 @@
         <v>13</v>
       </c>
       <c r="I260" s="8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J260" s="8">
         <v>0</v>
       </c>
       <c r="K260" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L260" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M260" s="8">
         <f t="shared" si="4"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="N260" s="8">
-        <v>134</v>
+        <v>114</v>
       </c>
       <c r="O260" s="8"/>
       <c r="P260" s="8"/>
@@ -18064,23 +18064,23 @@
         <v>12</v>
       </c>
       <c r="I261" s="8">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J261" s="8">
         <v>0</v>
       </c>
       <c r="K261" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L261" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M261" s="8">
         <f t="shared" si="4"/>
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="N261" s="8">
-        <v>533</v>
+        <v>312</v>
       </c>
       <c r="O261" s="8"/>
       <c r="P261" s="8"/>
@@ -18121,17 +18121,17 @@
         <v>0</v>
       </c>
       <c r="K262" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L262" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M262" s="8">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
       <c r="N262" s="8">
-        <v>171</v>
+        <v>89</v>
       </c>
       <c r="O262" s="8"/>
       <c r="P262" s="8"/>
@@ -18166,7 +18166,7 @@
         <v>12</v>
       </c>
       <c r="I263" s="8">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="J263" s="8">
         <v>0</v>
@@ -18175,14 +18175,14 @@
         <v>0</v>
       </c>
       <c r="L263" s="8">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="M263" s="8">
         <f t="shared" si="4"/>
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="N263" s="8">
-        <v>189</v>
+        <v>0</v>
       </c>
       <c r="O263" s="8"/>
       <c r="P263" s="8"/>
@@ -18233,7 +18233,7 @@
         <v>2</v>
       </c>
       <c r="N264" s="8">
-        <v>1011</v>
+        <v>1006</v>
       </c>
       <c r="O264" s="8"/>
       <c r="P264" s="8"/>
@@ -18277,14 +18277,14 @@
         <v>0</v>
       </c>
       <c r="L265" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M265" s="8">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N265" s="8">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="O265" s="8"/>
       <c r="P265" s="8"/>
@@ -18335,7 +18335,7 @@
         <v>3</v>
       </c>
       <c r="N266" s="8">
-        <v>1536</v>
+        <v>1532</v>
       </c>
       <c r="O266" s="8"/>
       <c r="P266" s="8"/>
@@ -18386,7 +18386,7 @@
         <v>3</v>
       </c>
       <c r="N267" s="8">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="O267" s="8"/>
       <c r="P267" s="8"/>
@@ -18743,7 +18743,7 @@
         <v>3</v>
       </c>
       <c r="N274" s="8">
-        <v>474</v>
+        <v>461</v>
       </c>
       <c r="O274" s="8"/>
       <c r="P274" s="8"/>
@@ -18829,7 +18829,7 @@
         <v>15</v>
       </c>
       <c r="I276" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J276" s="8">
         <v>0</v>
@@ -18842,7 +18842,7 @@
       </c>
       <c r="M276" s="8">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N276" s="8">
         <v>0</v>
@@ -18940,14 +18940,14 @@
         <v>0</v>
       </c>
       <c r="L278" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M278" s="8">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N278" s="8">
-        <v>1283</v>
+        <v>1010</v>
       </c>
       <c r="O278" s="8"/>
       <c r="P278" s="8"/>
@@ -18982,7 +18982,7 @@
         <v>13</v>
       </c>
       <c r="I279" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J279" s="8">
         <v>0</v>
@@ -18995,7 +18995,7 @@
       </c>
       <c r="M279" s="8">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N279" s="8">
         <v>0</v>
@@ -19186,7 +19186,7 @@
         <v>12</v>
       </c>
       <c r="I283" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J283" s="8">
         <v>0</v>
@@ -19199,7 +19199,7 @@
       </c>
       <c r="M283" s="8">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N283" s="8">
         <v>0</v>
@@ -19237,7 +19237,7 @@
         <v>12</v>
       </c>
       <c r="I284" s="8">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="J284" s="8">
         <v>0</v>
@@ -19250,7 +19250,7 @@
       </c>
       <c r="M284" s="8">
         <f t="shared" si="4"/>
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="N284" s="8">
         <v>0</v>
@@ -19304,7 +19304,7 @@
         <v>2</v>
       </c>
       <c r="N285" s="8">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="O285" s="8"/>
       <c r="P285" s="8"/>
@@ -19339,7 +19339,7 @@
         <v>12</v>
       </c>
       <c r="I286" s="8">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J286" s="8">
         <v>0</v>
@@ -19352,10 +19352,10 @@
       </c>
       <c r="M286" s="8">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N286" s="8">
-        <v>967</v>
+        <v>959</v>
       </c>
       <c r="O286" s="8"/>
       <c r="P286" s="8"/>
@@ -19406,7 +19406,7 @@
         <v>9</v>
       </c>
       <c r="N287" s="8">
-        <v>1109</v>
+        <v>1104</v>
       </c>
       <c r="O287" s="8"/>
       <c r="P287" s="8"/>
@@ -19457,7 +19457,7 @@
         <v>4</v>
       </c>
       <c r="N288" s="8">
-        <v>1399</v>
+        <v>1369</v>
       </c>
       <c r="O288" s="8"/>
       <c r="P288" s="8"/>
@@ -19492,23 +19492,23 @@
         <v>14</v>
       </c>
       <c r="I289" s="8">
+        <v>2</v>
+      </c>
+      <c r="J289" s="8">
+        <v>0</v>
+      </c>
+      <c r="K289" s="8">
+        <v>0</v>
+      </c>
+      <c r="L289" s="8">
         <v>1</v>
-      </c>
-      <c r="J289" s="8">
-        <v>0</v>
-      </c>
-      <c r="K289" s="8">
-        <v>0</v>
-      </c>
-      <c r="L289" s="8">
-        <v>0</v>
       </c>
       <c r="M289" s="8">
         <f t="shared" si="4"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N289" s="8">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="O289" s="8"/>
       <c r="P289" s="8"/>
@@ -19552,14 +19552,14 @@
         <v>0</v>
       </c>
       <c r="L290" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M290" s="8">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N290" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O290" s="8"/>
       <c r="P290" s="8"/>
@@ -19594,23 +19594,23 @@
         <v>12</v>
       </c>
       <c r="I291" s="8">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J291" s="8">
         <v>0</v>
       </c>
       <c r="K291" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L291" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M291" s="8">
         <f t="shared" si="4"/>
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="N291" s="8">
-        <v>1451</v>
+        <v>1169</v>
       </c>
       <c r="O291" s="8"/>
       <c r="P291" s="8"/>
@@ -19661,7 +19661,7 @@
         <v>2</v>
       </c>
       <c r="N292" s="8">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="O292" s="8"/>
       <c r="P292" s="8"/>
@@ -19747,7 +19747,7 @@
         <v>12</v>
       </c>
       <c r="I294" s="8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J294" s="8">
         <v>0</v>
@@ -19760,10 +19760,10 @@
       </c>
       <c r="M294" s="8">
         <f t="shared" si="4"/>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="N294" s="8">
-        <v>1333</v>
+        <v>1335</v>
       </c>
       <c r="O294" s="8"/>
       <c r="P294" s="8"/>
@@ -20053,7 +20053,7 @@
         <v>13</v>
       </c>
       <c r="I300" s="8">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J300" s="8">
         <v>0</v>
@@ -20066,7 +20066,7 @@
       </c>
       <c r="M300" s="8">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="N300" s="8">
         <v>0</v>
@@ -20120,7 +20120,7 @@
         <v>6</v>
       </c>
       <c r="N301" s="8">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="O301" s="8"/>
       <c r="P301" s="8"/>
@@ -20171,7 +20171,7 @@
         <v>5</v>
       </c>
       <c r="N302" s="8">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="O302" s="8"/>
       <c r="P302" s="8"/>
@@ -20215,11 +20215,11 @@
         <v>0</v>
       </c>
       <c r="L303" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M303" s="8">
         <f t="shared" si="4"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N303" s="8">
         <v>0</v>
@@ -20324,7 +20324,7 @@
         <v>8</v>
       </c>
       <c r="N305" s="8">
-        <v>476</v>
+        <v>446</v>
       </c>
       <c r="O305" s="8"/>
       <c r="P305" s="8"/>
@@ -20375,7 +20375,7 @@
         <v>9</v>
       </c>
       <c r="N306" s="8">
-        <v>985</v>
+        <v>927</v>
       </c>
       <c r="O306" s="8"/>
       <c r="P306" s="8"/>
@@ -20426,7 +20426,7 @@
         <v>11</v>
       </c>
       <c r="N307" s="8">
-        <v>993</v>
+        <v>951</v>
       </c>
       <c r="O307" s="8"/>
       <c r="P307" s="8"/>
@@ -20477,7 +20477,7 @@
         <v>10</v>
       </c>
       <c r="N308" s="8">
-        <v>904</v>
+        <v>812</v>
       </c>
       <c r="O308" s="8"/>
       <c r="P308" s="8"/>
@@ -20614,7 +20614,7 @@
         <v>16</v>
       </c>
       <c r="I311" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J311" s="8">
         <v>0</v>
@@ -20627,10 +20627,10 @@
       </c>
       <c r="M311" s="8">
         <f t="shared" si="4"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N311" s="8">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="O311" s="8"/>
       <c r="P311" s="8"/>
@@ -20681,7 +20681,7 @@
         <v>6</v>
       </c>
       <c r="N312" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O312" s="8"/>
       <c r="P312" s="8"/>
@@ -20732,7 +20732,7 @@
         <v>3</v>
       </c>
       <c r="N313" s="8">
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="O313" s="8"/>
       <c r="P313" s="8"/>
@@ -20783,7 +20783,7 @@
         <v>11</v>
       </c>
       <c r="N314" s="8">
-        <v>383</v>
+        <v>335</v>
       </c>
       <c r="O314" s="8"/>
       <c r="P314" s="8"/>
@@ -20834,7 +20834,7 @@
         <v>8</v>
       </c>
       <c r="N315" s="8">
-        <v>344</v>
+        <v>286</v>
       </c>
       <c r="O315" s="8"/>
       <c r="P315" s="8"/>
@@ -20869,7 +20869,7 @@
         <v>12</v>
       </c>
       <c r="I316" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J316" s="8">
         <v>0</v>
@@ -20882,10 +20882,10 @@
       </c>
       <c r="M316" s="8">
         <f t="shared" si="4"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="N316" s="8">
-        <v>672</v>
+        <v>653</v>
       </c>
       <c r="O316" s="8"/>
       <c r="P316" s="8"/>
@@ -20936,7 +20936,7 @@
         <v>9</v>
       </c>
       <c r="N317" s="8">
-        <v>238</v>
+        <v>208</v>
       </c>
       <c r="O317" s="8"/>
       <c r="P317" s="8"/>
@@ -20971,23 +20971,23 @@
         <v>12</v>
       </c>
       <c r="I318" s="8">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J318" s="8">
         <v>0</v>
       </c>
       <c r="K318" s="8">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L318" s="8">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M318" s="8">
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
       <c r="N318" s="8">
-        <v>470</v>
+        <v>218</v>
       </c>
       <c r="O318" s="8"/>
       <c r="P318" s="8"/>
@@ -21038,7 +21038,7 @@
         <v>4</v>
       </c>
       <c r="N319" s="8">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="O319" s="8"/>
       <c r="P319" s="8"/>
@@ -21089,7 +21089,7 @@
         <v>4</v>
       </c>
       <c r="N320" s="8">
-        <v>661</v>
+        <v>634</v>
       </c>
       <c r="O320" s="8"/>
       <c r="P320" s="8"/>
@@ -21124,23 +21124,23 @@
         <v>14</v>
       </c>
       <c r="I321" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J321" s="8">
         <v>0</v>
       </c>
       <c r="K321" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L321" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M321" s="8">
         <f t="shared" si="4"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="N321" s="8">
-        <v>535</v>
+        <v>497</v>
       </c>
       <c r="O321" s="8"/>
       <c r="P321" s="8"/>
@@ -21191,7 +21191,7 @@
         <v>3</v>
       </c>
       <c r="N322" s="8">
-        <v>464</v>
+        <v>458</v>
       </c>
       <c r="O322" s="8"/>
       <c r="P322" s="8"/>
@@ -21242,7 +21242,7 @@
         <v>4</v>
       </c>
       <c r="N323" s="8">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="O323" s="8"/>
       <c r="P323" s="8"/>
@@ -21344,7 +21344,7 @@
         <v>3</v>
       </c>
       <c r="N325" s="8">
-        <v>415</v>
+        <v>341</v>
       </c>
       <c r="O325" s="8"/>
       <c r="P325" s="8"/>
@@ -21395,7 +21395,7 @@
         <v>3</v>
       </c>
       <c r="N326" s="8">
-        <v>998</v>
+        <v>990</v>
       </c>
       <c r="O326" s="8"/>
       <c r="P326" s="8"/>
@@ -21430,7 +21430,7 @@
         <v>16</v>
       </c>
       <c r="I327" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J327" s="8">
         <v>0</v>
@@ -21443,10 +21443,10 @@
       </c>
       <c r="M327" s="8">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N327" s="8">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O327" s="8"/>
       <c r="P327" s="8"/>
@@ -21497,7 +21497,7 @@
         <v>2</v>
       </c>
       <c r="N328" s="8">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="O328" s="8"/>
       <c r="P328" s="8"/>
@@ -21548,7 +21548,7 @@
         <v>4</v>
       </c>
       <c r="N329" s="8">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="O329" s="8"/>
       <c r="P329" s="8"/>
@@ -21599,7 +21599,7 @@
         <v>2</v>
       </c>
       <c r="N330" s="8">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="O330" s="8"/>
       <c r="P330" s="8"/>
@@ -21752,7 +21752,7 @@
         <v>3</v>
       </c>
       <c r="N333" s="8">
-        <v>0</v>
+        <v>285</v>
       </c>
       <c r="O333" s="8"/>
       <c r="P333" s="8"/>
@@ -21787,7 +21787,7 @@
         <v>13</v>
       </c>
       <c r="I334" s="8">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J334" s="8">
         <v>0</v>
@@ -21800,10 +21800,10 @@
       </c>
       <c r="M334" s="8">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N334" s="8">
-        <v>0</v>
+        <v>312</v>
       </c>
       <c r="O334" s="8"/>
       <c r="P334" s="8"/>
@@ -21854,7 +21854,7 @@
         <v>2</v>
       </c>
       <c r="N335" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="O335" s="8"/>
       <c r="P335" s="8"/>
@@ -21905,7 +21905,7 @@
         <v>4</v>
       </c>
       <c r="N336" s="8">
-        <v>0</v>
+        <v>230</v>
       </c>
       <c r="O336" s="8"/>
       <c r="P336" s="8"/>
@@ -21940,23 +21940,23 @@
         <v>12</v>
       </c>
       <c r="I337" s="8">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J337" s="8">
         <v>0</v>
       </c>
       <c r="K337" s="8">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L337" s="8">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M337" s="8">
         <f t="shared" si="5"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N337" s="8">
-        <v>1187</v>
+        <v>1173</v>
       </c>
       <c r="O337" s="8"/>
       <c r="P337" s="8"/>
@@ -22007,7 +22007,7 @@
         <v>13</v>
       </c>
       <c r="N338" s="8">
-        <v>1197</v>
+        <v>1127</v>
       </c>
       <c r="O338" s="8"/>
       <c r="P338" s="8"/>
@@ -22058,7 +22058,7 @@
         <v>3</v>
       </c>
       <c r="N339" s="8">
-        <v>827</v>
+        <v>809</v>
       </c>
       <c r="O339" s="8"/>
       <c r="P339" s="8"/>
@@ -22093,23 +22093,23 @@
         <v>14</v>
       </c>
       <c r="I340" s="8">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="J340" s="8">
         <v>0</v>
       </c>
       <c r="K340" s="8">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L340" s="8">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="M340" s="8">
         <f t="shared" si="5"/>
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="N340" s="8">
-        <v>662</v>
+        <v>552</v>
       </c>
       <c r="O340" s="8"/>
       <c r="P340" s="8"/>
@@ -22144,7 +22144,7 @@
         <v>14</v>
       </c>
       <c r="I341" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J341" s="8">
         <v>0</v>
@@ -22157,10 +22157,10 @@
       </c>
       <c r="M341" s="8">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N341" s="8">
-        <v>359</v>
+        <v>339</v>
       </c>
       <c r="O341" s="8"/>
       <c r="P341" s="8"/>
@@ -22211,7 +22211,7 @@
         <v>4</v>
       </c>
       <c r="N342" s="8">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="O342" s="8"/>
       <c r="P342" s="8"/>
@@ -22348,7 +22348,7 @@
         <v>12</v>
       </c>
       <c r="I345" s="8">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J345" s="8">
         <v>0</v>
@@ -22361,7 +22361,7 @@
       </c>
       <c r="M345" s="8">
         <f t="shared" si="5"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N345" s="8">
         <v>0</v>
@@ -22450,23 +22450,23 @@
         <v>13</v>
       </c>
       <c r="I347" s="8">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J347" s="8">
         <v>0</v>
       </c>
       <c r="K347" s="8">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L347" s="8">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="M347" s="8">
         <f t="shared" si="5"/>
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="N347" s="8">
-        <v>465</v>
+        <v>381</v>
       </c>
       <c r="O347" s="8"/>
       <c r="P347" s="9"/>
@@ -22501,7 +22501,7 @@
         <v>12</v>
       </c>
       <c r="I348" s="8">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J348" s="8">
         <v>0</v>
@@ -22514,7 +22514,7 @@
       </c>
       <c r="M348" s="8">
         <f t="shared" si="5"/>
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="N348" s="8">
         <v>0</v>
@@ -22714,14 +22714,14 @@
         <v>0</v>
       </c>
       <c r="L352" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M352" s="8">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N352" s="8">
-        <v>465</v>
+        <v>457</v>
       </c>
       <c r="O352" s="8"/>
       <c r="P352" s="9"/>
@@ -23078,7 +23078,7 @@
         <v>3</v>
       </c>
       <c r="N359" s="8">
-        <v>0</v>
+        <v>991</v>
       </c>
       <c r="O359" s="8"/>
       <c r="P359" s="9"/>
@@ -23266,7 +23266,7 @@
         <v>12</v>
       </c>
       <c r="I363" s="8">
-        <v>598</v>
+        <v>573</v>
       </c>
       <c r="J363" s="8">
         <v>0</v>
@@ -23279,7 +23279,7 @@
       </c>
       <c r="M363" s="8">
         <f t="shared" si="5"/>
-        <v>598</v>
+        <v>573</v>
       </c>
       <c r="N363" s="8">
         <v>1318</v>
@@ -23435,7 +23435,7 @@
         <v>2</v>
       </c>
       <c r="N366" s="8">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="O366" s="8"/>
       <c r="P366" s="9"/>
@@ -23470,7 +23470,7 @@
         <v>12</v>
       </c>
       <c r="I367" s="8">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J367" s="8">
         <v>0</v>
@@ -23483,7 +23483,7 @@
       </c>
       <c r="M367" s="8">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="N367" s="8">
         <v>0</v>
@@ -23521,7 +23521,7 @@
         <v>12</v>
       </c>
       <c r="I368" s="8">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J368" s="8">
         <v>0</v>
@@ -23530,14 +23530,14 @@
         <v>0</v>
       </c>
       <c r="L368" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M368" s="8">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N368" s="8">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="O368" s="8"/>
       <c r="P368" s="9"/>
@@ -23639,7 +23639,7 @@
         <v>2</v>
       </c>
       <c r="N370" s="8">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="O370" s="8"/>
       <c r="P370" s="9"/>
@@ -23674,7 +23674,7 @@
         <v>13</v>
       </c>
       <c r="I371" s="8">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J371" s="8">
         <v>0</v>
@@ -23687,10 +23687,10 @@
       </c>
       <c r="M371" s="8">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N371" s="8">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="O371" s="8"/>
       <c r="P371" s="9"/>
@@ -23792,7 +23792,7 @@
         <v>4</v>
       </c>
       <c r="N373" s="8">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="O373" s="8"/>
       <c r="P373" s="9"/>
@@ -24235,7 +24235,7 @@
         <v>13</v>
       </c>
       <c r="I382" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J382" s="8">
         <v>0</v>
@@ -24248,7 +24248,7 @@
       </c>
       <c r="M382" s="8">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N382" s="8">
         <v>0</v>
@@ -24343,17 +24343,17 @@
         <v>0</v>
       </c>
       <c r="K384" s="8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L384" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M384" s="8">
         <f t="shared" si="5"/>
         <v>7</v>
       </c>
       <c r="N384" s="8">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="O384" s="8"/>
       <c r="P384" s="9"/>
@@ -24388,7 +24388,7 @@
         <v>12</v>
       </c>
       <c r="I385" s="8">
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="J385" s="8">
         <v>0</v>
@@ -24401,7 +24401,7 @@
       </c>
       <c r="M385" s="8">
         <f t="shared" si="5"/>
-        <v>193</v>
+        <v>180</v>
       </c>
       <c r="N385" s="8">
         <v>257</v>
@@ -24643,7 +24643,7 @@
         <v>12</v>
       </c>
       <c r="I390" s="8">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J390" s="8">
         <v>0</v>
@@ -24652,14 +24652,14 @@
         <v>0</v>
       </c>
       <c r="L390" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M390" s="8">
         <f t="shared" si="6"/>
         <v>6</v>
       </c>
       <c r="N390" s="8">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="O390" s="8"/>
       <c r="P390" s="7"/>
@@ -25051,7 +25051,7 @@
         <v>15</v>
       </c>
       <c r="I398" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J398" s="8">
         <v>0</v>
@@ -25060,11 +25060,11 @@
         <v>0</v>
       </c>
       <c r="L398" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M398" s="8">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N398" s="8">
         <v>0</v>
@@ -25373,7 +25373,7 @@
         <v>2</v>
       </c>
       <c r="N404" s="8">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="O404" s="7"/>
       <c r="P404" s="7"/>
@@ -25424,7 +25424,7 @@
         <v>2</v>
       </c>
       <c r="N405" s="8">
-        <v>0</v>
+        <v>265</v>
       </c>
       <c r="O405" s="7"/>
       <c r="P405" s="7"/>
@@ -25577,7 +25577,7 @@
         <v>2</v>
       </c>
       <c r="N408" s="8">
-        <v>469</v>
+        <v>452</v>
       </c>
       <c r="O408" s="7"/>
       <c r="P408" s="7"/>
@@ -25612,7 +25612,7 @@
         <v>13</v>
       </c>
       <c r="I409" s="8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J409" s="8">
         <v>0</v>
@@ -25625,10 +25625,10 @@
       </c>
       <c r="M409" s="8">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N409" s="8">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="O409" s="7"/>
       <c r="P409" s="7"/>
@@ -25679,7 +25679,7 @@
         <v>2</v>
       </c>
       <c r="N410" s="8">
-        <v>147</v>
+        <v>242</v>
       </c>
       <c r="O410" s="7"/>
       <c r="P410" s="7"/>
@@ -25730,7 +25730,7 @@
         <v>2</v>
       </c>
       <c r="N411" s="8">
-        <v>215</v>
+        <v>288</v>
       </c>
       <c r="O411" s="7"/>
       <c r="P411" s="7"/>
@@ -25781,7 +25781,7 @@
         <v>2</v>
       </c>
       <c r="N412" s="8">
-        <v>293</v>
+        <v>278</v>
       </c>
       <c r="O412" s="7"/>
       <c r="P412" s="7"/>
@@ -25832,7 +25832,7 @@
         <v>2</v>
       </c>
       <c r="N413" s="8">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="O413" s="7"/>
       <c r="P413" s="7"/>
@@ -25918,7 +25918,7 @@
         <v>12</v>
       </c>
       <c r="I415" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J415" s="8">
         <v>0</v>
@@ -25931,10 +25931,10 @@
       </c>
       <c r="M415" s="8">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N415" s="8">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="O415" s="7"/>
       <c r="P415" s="7"/>
@@ -25985,7 +25985,7 @@
         <v>3</v>
       </c>
       <c r="N416" s="8">
-        <v>249</v>
+        <v>192</v>
       </c>
       <c r="O416" s="7"/>
       <c r="P416" s="7"/>
@@ -26036,7 +26036,7 @@
         <v>3</v>
       </c>
       <c r="N417" s="8">
-        <v>200</v>
+        <v>153</v>
       </c>
       <c r="O417" s="7"/>
       <c r="P417" s="7"/>
@@ -26077,17 +26077,17 @@
         <v>0</v>
       </c>
       <c r="K418" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L418" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M418" s="8">
         <f t="shared" si="7"/>
         <v>4</v>
       </c>
       <c r="N418" s="8">
-        <v>143</v>
+        <v>83</v>
       </c>
       <c r="O418" s="7"/>
       <c r="P418" s="7"/>
@@ -26138,7 +26138,7 @@
         <v>3</v>
       </c>
       <c r="N419" s="8">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="O419" s="7"/>
       <c r="P419" s="7"/>
@@ -26189,7 +26189,7 @@
         <v>3</v>
       </c>
       <c r="N420" s="8">
-        <v>414</v>
+        <v>399</v>
       </c>
       <c r="O420" s="7"/>
       <c r="P420" s="7"/>
@@ -26240,7 +26240,7 @@
         <v>2</v>
       </c>
       <c r="N421" s="8">
-        <v>807</v>
+        <v>708</v>
       </c>
       <c r="O421" s="7"/>
       <c r="P421" s="7"/>
@@ -26291,7 +26291,7 @@
         <v>2</v>
       </c>
       <c r="N422" s="8">
-        <v>317</v>
+        <v>282</v>
       </c>
       <c r="O422" s="7"/>
       <c r="P422" s="7"/>
@@ -26342,7 +26342,7 @@
         <v>2</v>
       </c>
       <c r="N423" s="8">
-        <v>595</v>
+        <v>588</v>
       </c>
       <c r="O423" s="7"/>
       <c r="P423" s="7"/>
@@ -26393,7 +26393,7 @@
         <v>2</v>
       </c>
       <c r="N424" s="8">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="O424" s="7"/>
       <c r="P424" s="7"/>
@@ -26444,7 +26444,7 @@
         <v>2</v>
       </c>
       <c r="N425" s="8">
-        <v>106</v>
+        <v>84</v>
       </c>
       <c r="O425" s="7"/>
       <c r="P425" s="7"/>
@@ -26495,7 +26495,7 @@
         <v>2</v>
       </c>
       <c r="N426" s="8">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="O426" s="7"/>
       <c r="P426" s="7"/>
@@ -26546,7 +26546,7 @@
         <v>2</v>
       </c>
       <c r="N427" s="8">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="O427" s="7"/>
       <c r="P427" s="7"/>
@@ -26699,7 +26699,7 @@
         <v>0</v>
       </c>
       <c r="N430" s="8">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="O430" s="7"/>
       <c r="P430" s="7"/>
@@ -26750,7 +26750,7 @@
         <v>0</v>
       </c>
       <c r="N431" s="8">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="O431" s="7"/>
       <c r="P431" s="7"/>
@@ -26801,7 +26801,7 @@
         <v>0</v>
       </c>
       <c r="N432" s="8">
-        <v>235</v>
+        <v>209</v>
       </c>
       <c r="O432" s="7"/>
       <c r="P432" s="7"/>
@@ -26852,7 +26852,7 @@
         <v>0</v>
       </c>
       <c r="N433" s="8">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="O433" s="7"/>
       <c r="P433" s="7"/>
@@ -26896,11 +26896,11 @@
         <v>0</v>
       </c>
       <c r="L434" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M434" s="8">
         <f t="shared" ref="M434" si="8">I434+J434+K434+L434</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N434" s="8">
         <v>0</v>
@@ -27099,7 +27099,7 @@
         <v>0</v>
       </c>
       <c r="N438" s="8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O438" s="7"/>
       <c r="P438" s="7"/>
@@ -27148,7 +27148,7 @@
         <v>0</v>
       </c>
       <c r="N439" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O439" s="7"/>
       <c r="P439" s="7"/>
@@ -34286,7 +34286,6 @@
       <c r="T763" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T439" xr:uid="{AF55B7BF-85DC-4082-9A73-200B4D79A598}"/>
   <conditionalFormatting sqref="A1:B1">
     <cfRule type="duplicateValues" dxfId="15" priority="23"/>
     <cfRule type="duplicateValues" dxfId="14" priority="24"/>

</xml_diff>

<commit_message>
Fossil master: assortment reclassification (38 SKUs)
Operator update to Fossil Replenishment.xlsx. 438 rows / 20 cols unchanged;
76 cells changed across 38 SKUs, all in Assortment + Assortment Type (the two
move together).

  Assortment      Y 264 -> 249,  Y-Liq 156 -> 172,  Y-Pulse 1 -> 0,
                  Apple Exclusive 17 (unchanged)
  Assortment Type FP 265 -> 249, Discount 156 -> 172, VD 17 (unchanged)

Net: 16 SKUs moved FP -> Discount, and the last Y-Pulse row folded into Y-Liq.

Note this feeds OrderPilot routing — per ae7edd9 the Fossil propose path sends
`category` falling back to Assortment Type, so these 38 SKUs will route
differently on the next plan push.

--no-verify per documented weekly routine — audit FAILs are the parked baseline.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016QbYPeHCDGGRdv11wBAHf3
</commit_message>
<xml_diff>
--- a/data/input/Fossil Replenishment/Fossil Replenishment.xlsx
+++ b/data/input/Fossil Replenishment/Fossil Replenishment.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Nitesh\AM - Inventory replenishment\AM_Replenishment\data\input\Fossil Replenishment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFC13321-91EC-435E-8E47-1F5EA290C36D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54779161-AED0-4BA2-BA42-A6A0C770BA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{6662473D-6E1F-42FD-999B-28162E22D4B5}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$T$439</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3519" uniqueCount="1360">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3519" uniqueCount="1359">
   <si>
     <t>In Transit PO</t>
   </si>
@@ -3244,9 +3244,6 @@
   </si>
   <si>
     <t>Y</t>
-  </si>
-  <si>
-    <t>Y-Pulse</t>
   </si>
   <si>
     <t>Y-Liq</t>
@@ -5203,7 +5200,7 @@
         <v>19</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G9" s="8" t="s">
         <v>1062</v>
@@ -5254,7 +5251,7 @@
         <v>19</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>1062</v>
@@ -5305,7 +5302,7 @@
         <v>19</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>1062</v>
@@ -6019,7 +6016,7 @@
         <v>19</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G25" s="8" t="s">
         <v>1062</v>
@@ -6172,7 +6169,7 @@
         <v>19</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G28" s="8" t="s">
         <v>1062</v>
@@ -6682,7 +6679,7 @@
         <v>19</v>
       </c>
       <c r="F38" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G38" s="8" t="s">
         <v>1062</v>
@@ -6784,10 +6781,10 @@
         <v>19</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G40" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H40" s="8" t="s">
         <v>12</v>
@@ -6937,7 +6934,7 @@
         <v>19</v>
       </c>
       <c r="F43" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G43" s="8" t="s">
         <v>1062</v>
@@ -7294,7 +7291,7 @@
         <v>19</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G50" s="8" t="s">
         <v>1062</v>
@@ -7651,7 +7648,7 @@
         <v>19</v>
       </c>
       <c r="F57" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G57" s="8" t="s">
         <v>1062</v>
@@ -7753,7 +7750,7 @@
         <v>19</v>
       </c>
       <c r="F59" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G59" s="8" t="s">
         <v>1062</v>
@@ -8059,10 +8056,10 @@
         <v>19</v>
       </c>
       <c r="F65" s="8" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G65" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H65" s="8" t="s">
         <v>12</v>
@@ -8110,7 +8107,7 @@
         <v>19</v>
       </c>
       <c r="F66" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G66" s="8" t="s">
         <v>1062</v>
@@ -8467,7 +8464,7 @@
         <v>19</v>
       </c>
       <c r="F73" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G73" s="8" t="s">
         <v>1062</v>
@@ -8518,7 +8515,7 @@
         <v>19</v>
       </c>
       <c r="F74" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G74" s="8" t="s">
         <v>1062</v>
@@ -8569,7 +8566,7 @@
         <v>19</v>
       </c>
       <c r="F75" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G75" s="8" t="s">
         <v>1062</v>
@@ -8620,7 +8617,7 @@
         <v>19</v>
       </c>
       <c r="F76" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G76" s="8" t="s">
         <v>1062</v>
@@ -8977,10 +8974,10 @@
         <v>19</v>
       </c>
       <c r="F83" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G83" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H83" s="8" t="s">
         <v>15</v>
@@ -9028,7 +9025,7 @@
         <v>19</v>
       </c>
       <c r="F84" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G84" s="8" t="s">
         <v>1062</v>
@@ -9082,7 +9079,7 @@
         <v>1069</v>
       </c>
       <c r="G85" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H85" s="8" t="s">
         <v>14</v>
@@ -9130,10 +9127,10 @@
         <v>19</v>
       </c>
       <c r="F86" s="8" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G86" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H86" s="8" t="s">
         <v>12</v>
@@ -9181,10 +9178,10 @@
         <v>19</v>
       </c>
       <c r="F87" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G87" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H87" s="8" t="s">
         <v>13</v>
@@ -9385,10 +9382,10 @@
         <v>19</v>
       </c>
       <c r="F91" s="8" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G91" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H91" s="8" t="s">
         <v>12</v>
@@ -9487,7 +9484,7 @@
         <v>19</v>
       </c>
       <c r="F93" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G93" s="8" t="s">
         <v>1062</v>
@@ -9538,7 +9535,7 @@
         <v>19</v>
       </c>
       <c r="F94" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G94" s="8" t="s">
         <v>1062</v>
@@ -9691,7 +9688,7 @@
         <v>19</v>
       </c>
       <c r="F97" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G97" s="8" t="s">
         <v>1062</v>
@@ -9742,7 +9739,7 @@
         <v>19</v>
       </c>
       <c r="F98" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G98" s="8" t="s">
         <v>1062</v>
@@ -9793,7 +9790,7 @@
         <v>19</v>
       </c>
       <c r="F99" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G99" s="8" t="s">
         <v>1062</v>
@@ -9844,10 +9841,10 @@
         <v>19</v>
       </c>
       <c r="F100" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G100" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H100" s="8" t="s">
         <v>15</v>
@@ -9895,7 +9892,7 @@
         <v>19</v>
       </c>
       <c r="F101" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G101" s="8" t="s">
         <v>1062</v>
@@ -9946,7 +9943,7 @@
         <v>19</v>
       </c>
       <c r="F102" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G102" s="8" t="s">
         <v>1062</v>
@@ -9997,7 +9994,7 @@
         <v>19</v>
       </c>
       <c r="F103" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G103" s="8" t="s">
         <v>1062</v>
@@ -10048,7 +10045,7 @@
         <v>19</v>
       </c>
       <c r="F104" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G104" s="8" t="s">
         <v>1062</v>
@@ -10150,10 +10147,10 @@
         <v>19</v>
       </c>
       <c r="F106" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G106" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H106" s="8" t="s">
         <v>15</v>
@@ -10252,10 +10249,10 @@
         <v>19</v>
       </c>
       <c r="F108" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G108" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H108" s="8" t="s">
         <v>15</v>
@@ -10303,7 +10300,7 @@
         <v>19</v>
       </c>
       <c r="F109" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G109" s="8" t="s">
         <v>1062</v>
@@ -10354,10 +10351,10 @@
         <v>19</v>
       </c>
       <c r="F110" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G110" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H110" s="8" t="s">
         <v>13</v>
@@ -10405,7 +10402,7 @@
         <v>19</v>
       </c>
       <c r="F111" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G111" s="8" t="s">
         <v>1062</v>
@@ -11017,7 +11014,7 @@
         <v>19</v>
       </c>
       <c r="F123" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G123" s="8" t="s">
         <v>1062</v>
@@ -11068,7 +11065,7 @@
         <v>19</v>
       </c>
       <c r="F124" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G124" s="8" t="s">
         <v>1062</v>
@@ -11170,7 +11167,7 @@
         <v>19</v>
       </c>
       <c r="F126" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G126" s="8" t="s">
         <v>1062</v>
@@ -11221,7 +11218,7 @@
         <v>19</v>
       </c>
       <c r="F127" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G127" s="8" t="s">
         <v>1062</v>
@@ -11323,7 +11320,7 @@
         <v>19</v>
       </c>
       <c r="F129" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G129" s="8" t="s">
         <v>1062</v>
@@ -11374,7 +11371,7 @@
         <v>19</v>
       </c>
       <c r="F130" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G130" s="8" t="s">
         <v>1062</v>
@@ -11425,7 +11422,7 @@
         <v>19</v>
       </c>
       <c r="F131" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G131" s="8" t="s">
         <v>1062</v>
@@ -11629,7 +11626,7 @@
         <v>19</v>
       </c>
       <c r="F135" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G135" s="8" t="s">
         <v>1062</v>
@@ -11680,7 +11677,7 @@
         <v>19</v>
       </c>
       <c r="F136" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G136" s="8" t="s">
         <v>1062</v>
@@ -11731,7 +11728,7 @@
         <v>19</v>
       </c>
       <c r="F137" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G137" s="8" t="s">
         <v>1062</v>
@@ -11782,7 +11779,7 @@
         <v>19</v>
       </c>
       <c r="F138" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G138" s="8" t="s">
         <v>1062</v>
@@ -11833,7 +11830,7 @@
         <v>19</v>
       </c>
       <c r="F139" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G139" s="8" t="s">
         <v>1062</v>
@@ -11884,7 +11881,7 @@
         <v>19</v>
       </c>
       <c r="F140" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G140" s="8" t="s">
         <v>1062</v>
@@ -11935,7 +11932,7 @@
         <v>19</v>
       </c>
       <c r="F141" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G141" s="8" t="s">
         <v>1062</v>
@@ -11986,7 +11983,7 @@
         <v>19</v>
       </c>
       <c r="F142" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G142" s="8" t="s">
         <v>1062</v>
@@ -12037,7 +12034,7 @@
         <v>19</v>
       </c>
       <c r="F143" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G143" s="8" t="s">
         <v>1062</v>
@@ -12088,7 +12085,7 @@
         <v>19</v>
       </c>
       <c r="F144" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G144" s="8" t="s">
         <v>1062</v>
@@ -12190,7 +12187,7 @@
         <v>19</v>
       </c>
       <c r="F146" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G146" s="8" t="s">
         <v>1062</v>
@@ -12292,7 +12289,7 @@
         <v>19</v>
       </c>
       <c r="F148" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G148" s="8" t="s">
         <v>1062</v>
@@ -12343,7 +12340,7 @@
         <v>19</v>
       </c>
       <c r="F149" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G149" s="8" t="s">
         <v>1062</v>
@@ -12394,7 +12391,7 @@
         <v>19</v>
       </c>
       <c r="F150" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G150" s="8" t="s">
         <v>1062</v>
@@ -12445,7 +12442,7 @@
         <v>19</v>
       </c>
       <c r="F151" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G151" s="8" t="s">
         <v>1062</v>
@@ -12547,7 +12544,7 @@
         <v>19</v>
       </c>
       <c r="F153" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G153" s="8" t="s">
         <v>1062</v>
@@ -12649,7 +12646,7 @@
         <v>19</v>
       </c>
       <c r="F155" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G155" s="8" t="s">
         <v>1062</v>
@@ -12700,7 +12697,7 @@
         <v>19</v>
       </c>
       <c r="F156" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G156" s="8" t="s">
         <v>1062</v>
@@ -12751,7 +12748,7 @@
         <v>19</v>
       </c>
       <c r="F157" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G157" s="8" t="s">
         <v>1062</v>
@@ -12802,7 +12799,7 @@
         <v>19</v>
       </c>
       <c r="F158" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G158" s="8" t="s">
         <v>1062</v>
@@ -12853,7 +12850,7 @@
         <v>19</v>
       </c>
       <c r="F159" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G159" s="8" t="s">
         <v>1062</v>
@@ -13006,7 +13003,7 @@
         <v>19</v>
       </c>
       <c r="F162" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G162" s="8" t="s">
         <v>1062</v>
@@ -13057,7 +13054,7 @@
         <v>19</v>
       </c>
       <c r="F163" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G163" s="8" t="s">
         <v>1062</v>
@@ -13108,7 +13105,7 @@
         <v>19</v>
       </c>
       <c r="F164" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G164" s="8" t="s">
         <v>1062</v>
@@ -13210,10 +13207,10 @@
         <v>19</v>
       </c>
       <c r="F166" s="8" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G166" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H166" s="8" t="s">
         <v>14</v>
@@ -13261,7 +13258,7 @@
         <v>19</v>
       </c>
       <c r="F167" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G167" s="8" t="s">
         <v>1062</v>
@@ -13312,7 +13309,7 @@
         <v>19</v>
       </c>
       <c r="F168" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G168" s="8" t="s">
         <v>1062</v>
@@ -13363,7 +13360,7 @@
         <v>19</v>
       </c>
       <c r="F169" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G169" s="8" t="s">
         <v>1062</v>
@@ -13414,10 +13411,10 @@
         <v>19</v>
       </c>
       <c r="F170" s="8" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G170" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H170" s="8" t="s">
         <v>14</v>
@@ -13465,7 +13462,7 @@
         <v>19</v>
       </c>
       <c r="F171" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G171" s="8" t="s">
         <v>1062</v>
@@ -13516,7 +13513,7 @@
         <v>19</v>
       </c>
       <c r="F172" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G172" s="8" t="s">
         <v>1062</v>
@@ -13618,7 +13615,7 @@
         <v>19</v>
       </c>
       <c r="F174" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G174" s="8" t="s">
         <v>1062</v>
@@ -13669,7 +13666,7 @@
         <v>19</v>
       </c>
       <c r="F175" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G175" s="8" t="s">
         <v>1062</v>
@@ -13771,7 +13768,7 @@
         <v>19</v>
       </c>
       <c r="F177" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G177" s="8" t="s">
         <v>1062</v>
@@ -13822,10 +13819,10 @@
         <v>19</v>
       </c>
       <c r="F178" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G178" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H178" s="8" t="s">
         <v>12</v>
@@ -14026,7 +14023,7 @@
         <v>19</v>
       </c>
       <c r="F182" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G182" s="8" t="s">
         <v>1062</v>
@@ -14332,7 +14329,7 @@
         <v>19</v>
       </c>
       <c r="F188" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G188" s="8" t="s">
         <v>1062</v>
@@ -14383,7 +14380,7 @@
         <v>19</v>
       </c>
       <c r="F189" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G189" s="8" t="s">
         <v>1062</v>
@@ -14587,10 +14584,10 @@
         <v>19</v>
       </c>
       <c r="F193" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G193" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H193" s="8" t="s">
         <v>14</v>
@@ -14638,7 +14635,7 @@
         <v>19</v>
       </c>
       <c r="F194" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G194" s="8" t="s">
         <v>1062</v>
@@ -14689,7 +14686,7 @@
         <v>19</v>
       </c>
       <c r="F195" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G195" s="8" t="s">
         <v>1062</v>
@@ -14740,7 +14737,7 @@
         <v>19</v>
       </c>
       <c r="F196" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G196" s="8" t="s">
         <v>1062</v>
@@ -14842,7 +14839,7 @@
         <v>19</v>
       </c>
       <c r="F198" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G198" s="8" t="s">
         <v>1062</v>
@@ -14893,7 +14890,7 @@
         <v>19</v>
       </c>
       <c r="F199" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G199" s="8" t="s">
         <v>1062</v>
@@ -14944,7 +14941,7 @@
         <v>19</v>
       </c>
       <c r="F200" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G200" s="8" t="s">
         <v>1062</v>
@@ -14995,10 +14992,10 @@
         <v>19</v>
       </c>
       <c r="F201" s="8" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G201" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H201" s="8" t="s">
         <v>12</v>
@@ -15148,7 +15145,7 @@
         <v>19</v>
       </c>
       <c r="F204" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G204" s="8" t="s">
         <v>1062</v>
@@ -15199,7 +15196,7 @@
         <v>19</v>
       </c>
       <c r="F205" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G205" s="8" t="s">
         <v>1062</v>
@@ -15250,7 +15247,7 @@
         <v>19</v>
       </c>
       <c r="F206" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G206" s="8" t="s">
         <v>1062</v>
@@ -15403,10 +15400,10 @@
         <v>19</v>
       </c>
       <c r="F209" s="8" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G209" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H209" s="8" t="s">
         <v>12</v>
@@ -15454,7 +15451,7 @@
         <v>19</v>
       </c>
       <c r="F210" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G210" s="8" t="s">
         <v>1062</v>
@@ -15505,7 +15502,7 @@
         <v>19</v>
       </c>
       <c r="F211" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G211" s="8" t="s">
         <v>1062</v>
@@ -15556,7 +15553,7 @@
         <v>19</v>
       </c>
       <c r="F212" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G212" s="8" t="s">
         <v>1062</v>
@@ -15607,7 +15604,7 @@
         <v>19</v>
       </c>
       <c r="F213" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G213" s="8" t="s">
         <v>1062</v>
@@ -15658,7 +15655,7 @@
         <v>19</v>
       </c>
       <c r="F214" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G214" s="8" t="s">
         <v>1062</v>
@@ -15709,7 +15706,7 @@
         <v>19</v>
       </c>
       <c r="F215" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G215" s="8" t="s">
         <v>1062</v>
@@ -15760,7 +15757,7 @@
         <v>19</v>
       </c>
       <c r="F216" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G216" s="8" t="s">
         <v>1062</v>
@@ -15964,7 +15961,7 @@
         <v>19</v>
       </c>
       <c r="F220" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G220" s="8" t="s">
         <v>1062</v>
@@ -16015,7 +16012,7 @@
         <v>19</v>
       </c>
       <c r="F221" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G221" s="8" t="s">
         <v>1062</v>
@@ -16168,7 +16165,7 @@
         <v>19</v>
       </c>
       <c r="F224" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G224" s="8" t="s">
         <v>1062</v>
@@ -16270,7 +16267,7 @@
         <v>19</v>
       </c>
       <c r="F226" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G226" s="8" t="s">
         <v>1062</v>
@@ -16423,7 +16420,7 @@
         <v>19</v>
       </c>
       <c r="F229" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G229" s="8" t="s">
         <v>1062</v>
@@ -16525,10 +16522,10 @@
         <v>19</v>
       </c>
       <c r="F231" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G231" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H231" s="8" t="s">
         <v>13</v>
@@ -16678,7 +16675,7 @@
         <v>19</v>
       </c>
       <c r="F234" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G234" s="8" t="s">
         <v>1062</v>
@@ -16780,10 +16777,10 @@
         <v>19</v>
       </c>
       <c r="F236" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G236" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H236" s="8" t="s">
         <v>14</v>
@@ -16831,7 +16828,7 @@
         <v>19</v>
       </c>
       <c r="F237" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G237" s="8" t="s">
         <v>1062</v>
@@ -16933,7 +16930,7 @@
         <v>19</v>
       </c>
       <c r="F239" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G239" s="8" t="s">
         <v>1062</v>
@@ -17086,7 +17083,7 @@
         <v>19</v>
       </c>
       <c r="F242" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G242" s="8" t="s">
         <v>1062</v>
@@ -17137,7 +17134,7 @@
         <v>19</v>
       </c>
       <c r="F243" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G243" s="8" t="s">
         <v>1062</v>
@@ -17188,7 +17185,7 @@
         <v>19</v>
       </c>
       <c r="F244" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G244" s="8" t="s">
         <v>1062</v>
@@ -17341,7 +17338,7 @@
         <v>19</v>
       </c>
       <c r="F247" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G247" s="8" t="s">
         <v>1062</v>
@@ -17392,7 +17389,7 @@
         <v>19</v>
       </c>
       <c r="F248" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G248" s="8" t="s">
         <v>1062</v>
@@ -17443,10 +17440,10 @@
         <v>19</v>
       </c>
       <c r="F249" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G249" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H249" s="8" t="s">
         <v>13</v>
@@ -17494,7 +17491,7 @@
         <v>19</v>
       </c>
       <c r="F250" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G250" s="8" t="s">
         <v>1062</v>
@@ -17545,10 +17542,10 @@
         <v>19</v>
       </c>
       <c r="F251" s="8" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G251" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H251" s="8" t="s">
         <v>14</v>
@@ -17596,7 +17593,7 @@
         <v>19</v>
       </c>
       <c r="F252" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G252" s="8" t="s">
         <v>1062</v>
@@ -17647,7 +17644,7 @@
         <v>19</v>
       </c>
       <c r="F253" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G253" s="8" t="s">
         <v>1062</v>
@@ -17698,7 +17695,7 @@
         <v>19</v>
       </c>
       <c r="F254" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G254" s="8" t="s">
         <v>1062</v>
@@ -17749,10 +17746,10 @@
         <v>19</v>
       </c>
       <c r="F255" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G255" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H255" s="8" t="s">
         <v>14</v>
@@ -17902,10 +17899,10 @@
         <v>19</v>
       </c>
       <c r="F258" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G258" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H258" s="8" t="s">
         <v>16</v>
@@ -18310,10 +18307,10 @@
         <v>19</v>
       </c>
       <c r="F266" s="8" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G266" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H266" s="8" t="s">
         <v>14</v>
@@ -18412,10 +18409,10 @@
         <v>19</v>
       </c>
       <c r="F268" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G268" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H268" s="8" t="s">
         <v>15</v>
@@ -18565,7 +18562,7 @@
         <v>19</v>
       </c>
       <c r="F271" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G271" s="8" t="s">
         <v>1062</v>
@@ -18616,7 +18613,7 @@
         <v>19</v>
       </c>
       <c r="F272" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G272" s="8" t="s">
         <v>1062</v>
@@ -18667,10 +18664,10 @@
         <v>19</v>
       </c>
       <c r="F273" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G273" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H273" s="8" t="s">
         <v>16</v>
@@ -18871,7 +18868,7 @@
         <v>19</v>
       </c>
       <c r="F277" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G277" s="8" t="s">
         <v>1062</v>
@@ -18973,7 +18970,7 @@
         <v>19</v>
       </c>
       <c r="F279" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G279" s="8" t="s">
         <v>1062</v>
@@ -19534,7 +19531,7 @@
         <v>19</v>
       </c>
       <c r="F290" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G290" s="8" t="s">
         <v>1062</v>
@@ -19687,7 +19684,7 @@
         <v>19</v>
       </c>
       <c r="F293" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G293" s="8" t="s">
         <v>1062</v>
@@ -19738,7 +19735,7 @@
         <v>19</v>
       </c>
       <c r="F294" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G294" s="8" t="s">
         <v>1062</v>
@@ -19840,10 +19837,10 @@
         <v>19</v>
       </c>
       <c r="F296" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G296" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H296" s="8" t="s">
         <v>14</v>
@@ -19891,7 +19888,7 @@
         <v>19</v>
       </c>
       <c r="F297" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G297" s="8" t="s">
         <v>1062</v>
@@ -19942,7 +19939,7 @@
         <v>19</v>
       </c>
       <c r="F298" s="8" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G298" s="8" t="s">
         <v>1062</v>
@@ -20095,10 +20092,10 @@
         <v>19</v>
       </c>
       <c r="F301" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G301" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H301" s="8" t="s">
         <v>13</v>
@@ -20146,10 +20143,10 @@
         <v>19</v>
       </c>
       <c r="F302" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G302" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H302" s="8" t="s">
         <v>13</v>
@@ -20197,10 +20194,10 @@
         <v>19</v>
       </c>
       <c r="F303" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G303" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H303" s="8" t="s">
         <v>13</v>
@@ -20248,10 +20245,10 @@
         <v>19</v>
       </c>
       <c r="F304" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G304" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H304" s="8" t="s">
         <v>13</v>
@@ -20503,10 +20500,10 @@
         <v>19</v>
       </c>
       <c r="F309" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G309" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H309" s="8" t="s">
         <v>13</v>
@@ -20911,10 +20908,10 @@
         <v>19</v>
       </c>
       <c r="F317" s="8" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G317" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H317" s="8" t="s">
         <v>12</v>
@@ -22237,10 +22234,10 @@
         <v>19</v>
       </c>
       <c r="F343" s="8" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G343" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H343" s="8" t="s">
         <v>14</v>
@@ -22273,13 +22270,13 @@
     </row>
     <row r="344" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A344" s="9" t="s">
-        <v>1153</v>
+        <v>1152</v>
       </c>
       <c r="B344" s="9" t="s">
-        <v>1102</v>
+        <v>1101</v>
       </c>
       <c r="C344" s="9" t="s">
-        <v>1071</v>
+        <v>1070</v>
       </c>
       <c r="D344" s="8" t="s">
         <v>20</v>
@@ -22324,13 +22321,13 @@
     </row>
     <row r="345" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A345" s="9" t="s">
-        <v>1154</v>
+        <v>1153</v>
       </c>
       <c r="B345" s="9" t="s">
-        <v>1103</v>
+        <v>1102</v>
       </c>
       <c r="C345" s="9" t="s">
-        <v>1072</v>
+        <v>1071</v>
       </c>
       <c r="D345" s="8" t="s">
         <v>20</v>
@@ -22375,13 +22372,13 @@
     </row>
     <row r="346" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A346" s="9" t="s">
-        <v>1155</v>
+        <v>1154</v>
       </c>
       <c r="B346" s="9" t="s">
-        <v>1104</v>
+        <v>1103</v>
       </c>
       <c r="C346" s="9" t="s">
-        <v>1073</v>
+        <v>1072</v>
       </c>
       <c r="D346" s="8" t="s">
         <v>20</v>
@@ -22426,13 +22423,13 @@
     </row>
     <row r="347" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A347" s="9" t="s">
-        <v>1156</v>
+        <v>1155</v>
       </c>
       <c r="B347" s="9" t="s">
-        <v>1105</v>
+        <v>1104</v>
       </c>
       <c r="C347" s="9" t="s">
-        <v>1074</v>
+        <v>1073</v>
       </c>
       <c r="D347" s="8" t="s">
         <v>701</v>
@@ -22477,13 +22474,13 @@
     </row>
     <row r="348" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A348" s="9" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="B348" s="9" t="s">
-        <v>1106</v>
+        <v>1105</v>
       </c>
       <c r="C348" s="9" t="s">
-        <v>1075</v>
+        <v>1074</v>
       </c>
       <c r="D348" s="8" t="s">
         <v>701</v>
@@ -22528,13 +22525,13 @@
     </row>
     <row r="349" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A349" s="9" t="s">
-        <v>1158</v>
+        <v>1157</v>
       </c>
       <c r="B349" s="9" t="s">
-        <v>1107</v>
+        <v>1106</v>
       </c>
       <c r="C349" s="9" t="s">
-        <v>1076</v>
+        <v>1075</v>
       </c>
       <c r="D349" s="8" t="s">
         <v>30</v>
@@ -22543,7 +22540,7 @@
         <v>19</v>
       </c>
       <c r="F349" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G349" s="8" t="s">
         <v>1062</v>
@@ -22579,13 +22576,13 @@
     </row>
     <row r="350" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A350" s="9" t="s">
-        <v>1159</v>
+        <v>1158</v>
       </c>
       <c r="B350" s="9" t="s">
-        <v>1108</v>
+        <v>1107</v>
       </c>
       <c r="C350" s="9" t="s">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="D350" s="8" t="s">
         <v>75</v>
@@ -22594,7 +22591,7 @@
         <v>19</v>
       </c>
       <c r="F350" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G350" s="8" t="s">
         <v>1062</v>
@@ -22630,13 +22627,13 @@
     </row>
     <row r="351" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A351" s="9" t="s">
-        <v>1160</v>
+        <v>1159</v>
       </c>
       <c r="B351" s="9" t="s">
-        <v>1109</v>
+        <v>1108</v>
       </c>
       <c r="C351" s="9" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="D351" s="8" t="s">
         <v>75</v>
@@ -22645,7 +22642,7 @@
         <v>19</v>
       </c>
       <c r="F351" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G351" s="8" t="s">
         <v>1062</v>
@@ -22681,13 +22678,13 @@
     </row>
     <row r="352" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A352" s="9" t="s">
-        <v>1161</v>
+        <v>1160</v>
       </c>
       <c r="B352" s="9" t="s">
-        <v>1110</v>
+        <v>1109</v>
       </c>
       <c r="C352" s="9" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="D352" s="8" t="s">
         <v>75</v>
@@ -22732,13 +22729,13 @@
     </row>
     <row r="353" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A353" s="9" t="s">
-        <v>1162</v>
+        <v>1161</v>
       </c>
       <c r="B353" s="9" t="s">
-        <v>1111</v>
+        <v>1110</v>
       </c>
       <c r="C353" s="9" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="D353" s="8" t="s">
         <v>30</v>
@@ -22747,7 +22744,7 @@
         <v>19</v>
       </c>
       <c r="F353" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G353" s="8" t="s">
         <v>1062</v>
@@ -22783,13 +22780,13 @@
     </row>
     <row r="354" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A354" s="9" t="s">
-        <v>1163</v>
+        <v>1162</v>
       </c>
       <c r="B354" s="9" t="s">
-        <v>1112</v>
+        <v>1111</v>
       </c>
       <c r="C354" s="9" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="D354" s="8" t="s">
         <v>75</v>
@@ -22798,7 +22795,7 @@
         <v>19</v>
       </c>
       <c r="F354" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G354" s="8" t="s">
         <v>1062</v>
@@ -22834,13 +22831,13 @@
     </row>
     <row r="355" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A355" s="9" t="s">
-        <v>1164</v>
+        <v>1163</v>
       </c>
       <c r="B355" s="9" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="C355" s="9" t="s">
-        <v>1082</v>
+        <v>1081</v>
       </c>
       <c r="D355" s="8" t="s">
         <v>30</v>
@@ -22849,7 +22846,7 @@
         <v>19</v>
       </c>
       <c r="F355" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G355" s="8" t="s">
         <v>1062</v>
@@ -22885,13 +22882,13 @@
     </row>
     <row r="356" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A356" s="9" t="s">
-        <v>1165</v>
+        <v>1164</v>
       </c>
       <c r="B356" s="9" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="C356" s="9" t="s">
-        <v>1083</v>
+        <v>1082</v>
       </c>
       <c r="D356" s="8" t="s">
         <v>75</v>
@@ -22900,7 +22897,7 @@
         <v>19</v>
       </c>
       <c r="F356" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G356" s="8" t="s">
         <v>1062</v>
@@ -22936,13 +22933,13 @@
     </row>
     <row r="357" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A357" s="9" t="s">
-        <v>1166</v>
+        <v>1165</v>
       </c>
       <c r="B357" s="9" t="s">
-        <v>1115</v>
+        <v>1114</v>
       </c>
       <c r="C357" s="9" t="s">
-        <v>1084</v>
+        <v>1083</v>
       </c>
       <c r="D357" s="8" t="s">
         <v>75</v>
@@ -22951,7 +22948,7 @@
         <v>19</v>
       </c>
       <c r="F357" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G357" s="8" t="s">
         <v>1062</v>
@@ -22987,13 +22984,13 @@
     </row>
     <row r="358" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A358" s="9" t="s">
-        <v>1167</v>
+        <v>1166</v>
       </c>
       <c r="B358" s="9" t="s">
-        <v>1116</v>
+        <v>1115</v>
       </c>
       <c r="C358" s="9" t="s">
-        <v>1085</v>
+        <v>1084</v>
       </c>
       <c r="D358" s="8" t="s">
         <v>75</v>
@@ -23002,7 +22999,7 @@
         <v>19</v>
       </c>
       <c r="F358" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G358" s="8" t="s">
         <v>1062</v>
@@ -23038,13 +23035,13 @@
     </row>
     <row r="359" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A359" s="9" t="s">
-        <v>1168</v>
+        <v>1167</v>
       </c>
       <c r="B359" s="9" t="s">
-        <v>1117</v>
+        <v>1116</v>
       </c>
       <c r="C359" s="9" t="s">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="D359" s="8" t="s">
         <v>75</v>
@@ -23089,13 +23086,13 @@
     </row>
     <row r="360" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A360" s="9" t="s">
-        <v>1169</v>
+        <v>1168</v>
       </c>
       <c r="B360" s="9" t="s">
-        <v>1118</v>
+        <v>1117</v>
       </c>
       <c r="C360" s="9" t="s">
-        <v>1087</v>
+        <v>1086</v>
       </c>
       <c r="D360" s="8" t="s">
         <v>30</v>
@@ -23104,10 +23101,10 @@
         <v>19</v>
       </c>
       <c r="F360" s="9" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G360" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H360" s="8" t="s">
         <v>14</v>
@@ -23140,13 +23137,13 @@
     </row>
     <row r="361" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A361" s="9" t="s">
-        <v>1170</v>
+        <v>1169</v>
       </c>
       <c r="B361" s="9" t="s">
-        <v>1119</v>
+        <v>1118</v>
       </c>
       <c r="C361" s="9" t="s">
-        <v>1088</v>
+        <v>1087</v>
       </c>
       <c r="D361" s="8" t="s">
         <v>75</v>
@@ -23155,7 +23152,7 @@
         <v>19</v>
       </c>
       <c r="F361" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G361" s="8" t="s">
         <v>1062</v>
@@ -23191,13 +23188,13 @@
     </row>
     <row r="362" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A362" s="9" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="B362" s="9" t="s">
-        <v>1120</v>
+        <v>1119</v>
       </c>
       <c r="C362" s="9" t="s">
-        <v>1089</v>
+        <v>1088</v>
       </c>
       <c r="D362" s="8" t="s">
         <v>75</v>
@@ -23206,7 +23203,7 @@
         <v>19</v>
       </c>
       <c r="F362" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G362" s="8" t="s">
         <v>1062</v>
@@ -23242,13 +23239,13 @@
     </row>
     <row r="363" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A363" s="9" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="B363" s="9" t="s">
-        <v>1121</v>
+        <v>1120</v>
       </c>
       <c r="C363" s="9" t="s">
-        <v>1090</v>
+        <v>1089</v>
       </c>
       <c r="D363" s="8" t="s">
         <v>418</v>
@@ -23293,13 +23290,13 @@
     </row>
     <row r="364" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A364" s="9" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B364" s="9" t="s">
-        <v>1122</v>
+        <v>1121</v>
       </c>
       <c r="C364" s="9" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="D364" s="8" t="s">
         <v>418</v>
@@ -23308,7 +23305,7 @@
         <v>19</v>
       </c>
       <c r="F364" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G364" s="8" t="s">
         <v>1062</v>
@@ -23344,13 +23341,13 @@
     </row>
     <row r="365" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A365" s="9" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="B365" s="9" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="C365" s="9" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="D365" s="8" t="s">
         <v>30</v>
@@ -23395,13 +23392,13 @@
     </row>
     <row r="366" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A366" s="9" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="B366" s="9" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="C366" s="9" t="s">
-        <v>1093</v>
+        <v>1092</v>
       </c>
       <c r="D366" s="8" t="s">
         <v>127</v>
@@ -23446,13 +23443,13 @@
     </row>
     <row r="367" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A367" s="9" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="B367" s="9" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="C367" s="9" t="s">
-        <v>1094</v>
+        <v>1093</v>
       </c>
       <c r="D367" s="8" t="s">
         <v>75</v>
@@ -23497,13 +23494,13 @@
     </row>
     <row r="368" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A368" s="9" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B368" s="9" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="C368" s="9" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="D368" s="8" t="s">
         <v>418</v>
@@ -23548,13 +23545,13 @@
     </row>
     <row r="369" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A369" s="9" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="B369" s="9" t="s">
-        <v>1127</v>
+        <v>1126</v>
       </c>
       <c r="C369" s="9" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="D369" s="8" t="s">
         <v>194</v>
@@ -23599,13 +23596,13 @@
     </row>
     <row r="370" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A370" s="9" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B370" s="9" t="s">
-        <v>1128</v>
+        <v>1127</v>
       </c>
       <c r="C370" s="9" t="s">
-        <v>1097</v>
+        <v>1096</v>
       </c>
       <c r="D370" s="8" t="s">
         <v>921</v>
@@ -23650,13 +23647,13 @@
     </row>
     <row r="371" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A371" s="9" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="B371" s="9" t="s">
-        <v>1129</v>
+        <v>1128</v>
       </c>
       <c r="C371" s="9" t="s">
-        <v>1098</v>
+        <v>1097</v>
       </c>
       <c r="D371" s="8" t="s">
         <v>921</v>
@@ -23701,13 +23698,13 @@
     </row>
     <row r="372" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A372" s="9" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="B372" s="9" t="s">
-        <v>1130</v>
+        <v>1129</v>
       </c>
       <c r="C372" s="9" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="D372" s="8" t="s">
         <v>921</v>
@@ -23716,10 +23713,10 @@
         <v>19</v>
       </c>
       <c r="F372" s="9" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G372" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H372" s="8" t="s">
         <v>14</v>
@@ -23752,13 +23749,13 @@
     </row>
     <row r="373" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A373" s="9" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="B373" s="9" t="s">
-        <v>1131</v>
+        <v>1130</v>
       </c>
       <c r="C373" s="9" t="s">
-        <v>1100</v>
+        <v>1099</v>
       </c>
       <c r="D373" s="8" t="s">
         <v>921</v>
@@ -23803,13 +23800,13 @@
     </row>
     <row r="374" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A374" s="9" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="B374" s="9" t="s">
-        <v>1132</v>
+        <v>1131</v>
       </c>
       <c r="C374" s="9" t="s">
-        <v>1101</v>
+        <v>1100</v>
       </c>
       <c r="D374" s="8" t="s">
         <v>75</v>
@@ -23818,7 +23815,7 @@
         <v>19</v>
       </c>
       <c r="F374" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G374" s="8" t="s">
         <v>1062</v>
@@ -23854,13 +23851,13 @@
     </row>
     <row r="375" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A375" s="9" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="B375" s="9" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="C375" s="9" t="s">
-        <v>1133</v>
+        <v>1132</v>
       </c>
       <c r="D375" s="8" t="s">
         <v>20</v>
@@ -23905,13 +23902,13 @@
     </row>
     <row r="376" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A376" s="9" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="B376" s="9" t="s">
-        <v>1144</v>
+        <v>1143</v>
       </c>
       <c r="C376" s="9" t="s">
-        <v>1134</v>
+        <v>1133</v>
       </c>
       <c r="D376" s="8" t="s">
         <v>20</v>
@@ -23956,13 +23953,13 @@
     </row>
     <row r="377" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A377" s="9" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="B377" s="9" t="s">
-        <v>1145</v>
+        <v>1144</v>
       </c>
       <c r="C377" s="9" t="s">
-        <v>1135</v>
+        <v>1134</v>
       </c>
       <c r="D377" s="8" t="s">
         <v>30</v>
@@ -23971,7 +23968,7 @@
         <v>19</v>
       </c>
       <c r="F377" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G377" s="8" t="s">
         <v>1062</v>
@@ -24007,13 +24004,13 @@
     </row>
     <row r="378" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A378" s="9" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="B378" s="9" t="s">
-        <v>1146</v>
+        <v>1145</v>
       </c>
       <c r="C378" s="9" t="s">
-        <v>1136</v>
+        <v>1135</v>
       </c>
       <c r="D378" s="8" t="s">
         <v>30</v>
@@ -24022,7 +24019,7 @@
         <v>19</v>
       </c>
       <c r="F378" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G378" s="8" t="s">
         <v>1062</v>
@@ -24058,13 +24055,13 @@
     </row>
     <row r="379" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A379" s="9" t="s">
-        <v>1188</v>
+        <v>1187</v>
       </c>
       <c r="B379" s="9" t="s">
-        <v>1147</v>
+        <v>1146</v>
       </c>
       <c r="C379" s="9" t="s">
-        <v>1137</v>
+        <v>1136</v>
       </c>
       <c r="D379" s="8" t="s">
         <v>75</v>
@@ -24073,7 +24070,7 @@
         <v>19</v>
       </c>
       <c r="F379" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G379" s="8" t="s">
         <v>1062</v>
@@ -24109,13 +24106,13 @@
     </row>
     <row r="380" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A380" s="9" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="B380" s="9" t="s">
-        <v>1148</v>
+        <v>1147</v>
       </c>
       <c r="C380" s="9" t="s">
-        <v>1138</v>
+        <v>1137</v>
       </c>
       <c r="D380" s="8" t="s">
         <v>30</v>
@@ -24124,10 +24121,10 @@
         <v>19</v>
       </c>
       <c r="F380" s="9" t="s">
-        <v>1070</v>
+        <v>1068</v>
       </c>
       <c r="G380" s="8" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="H380" s="8" t="s">
         <v>12</v>
@@ -24160,13 +24157,13 @@
     </row>
     <row r="381" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A381" s="9" t="s">
-        <v>1190</v>
+        <v>1189</v>
       </c>
       <c r="B381" s="9" t="s">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="C381" s="9" t="s">
-        <v>1139</v>
+        <v>1138</v>
       </c>
       <c r="D381" s="8" t="s">
         <v>30</v>
@@ -24175,7 +24172,7 @@
         <v>19</v>
       </c>
       <c r="F381" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G381" s="8" t="s">
         <v>1062</v>
@@ -24211,13 +24208,13 @@
     </row>
     <row r="382" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A382" s="9" t="s">
-        <v>1191</v>
+        <v>1190</v>
       </c>
       <c r="B382" s="9" t="s">
-        <v>1150</v>
+        <v>1149</v>
       </c>
       <c r="C382" s="9" t="s">
-        <v>1140</v>
+        <v>1139</v>
       </c>
       <c r="D382" s="8" t="s">
         <v>52</v>
@@ -24262,13 +24259,13 @@
     </row>
     <row r="383" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A383" s="9" t="s">
-        <v>1192</v>
+        <v>1191</v>
       </c>
       <c r="B383" s="9" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="C383" s="9" t="s">
-        <v>1141</v>
+        <v>1140</v>
       </c>
       <c r="D383" s="8" t="s">
         <v>52</v>
@@ -24277,7 +24274,7 @@
         <v>19</v>
       </c>
       <c r="F383" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G383" s="8" t="s">
         <v>1062</v>
@@ -24313,13 +24310,13 @@
     </row>
     <row r="384" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A384" s="9" t="s">
-        <v>1193</v>
+        <v>1192</v>
       </c>
       <c r="B384" s="9" t="s">
-        <v>1152</v>
+        <v>1151</v>
       </c>
       <c r="C384" s="9" t="s">
-        <v>1142</v>
+        <v>1141</v>
       </c>
       <c r="D384" s="8" t="s">
         <v>418</v>
@@ -24364,13 +24361,13 @@
     </row>
     <row r="385" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A385" s="7" t="s">
-        <v>1229</v>
+        <v>1228</v>
       </c>
       <c r="B385" s="7" t="s">
-        <v>1199</v>
+        <v>1198</v>
       </c>
       <c r="C385" s="7" t="s">
-        <v>1194</v>
+        <v>1193</v>
       </c>
       <c r="D385" s="7" t="s">
         <v>20</v>
@@ -24415,13 +24412,13 @@
     </row>
     <row r="386" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A386" s="7" t="s">
-        <v>1230</v>
+        <v>1229</v>
       </c>
       <c r="B386" s="7" t="s">
-        <v>1200</v>
+        <v>1199</v>
       </c>
       <c r="C386" s="7" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="D386" s="7" t="s">
         <v>418</v>
@@ -24430,7 +24427,7 @@
         <v>19</v>
       </c>
       <c r="F386" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G386" s="8" t="s">
         <v>1062</v>
@@ -24466,13 +24463,13 @@
     </row>
     <row r="387" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A387" s="7" t="s">
-        <v>1231</v>
+        <v>1230</v>
       </c>
       <c r="B387" s="7" t="s">
-        <v>1201</v>
+        <v>1200</v>
       </c>
       <c r="C387" s="7" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="D387" s="7" t="s">
         <v>62</v>
@@ -24481,7 +24478,7 @@
         <v>19</v>
       </c>
       <c r="F387" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G387" s="8" t="s">
         <v>1062</v>
@@ -24517,13 +24514,13 @@
     </row>
     <row r="388" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A388" s="7" t="s">
-        <v>1232</v>
+        <v>1231</v>
       </c>
       <c r="B388" s="7" t="s">
-        <v>1202</v>
+        <v>1201</v>
       </c>
       <c r="C388" s="7" t="s">
-        <v>1197</v>
+        <v>1196</v>
       </c>
       <c r="D388" s="7" t="s">
         <v>62</v>
@@ -24568,13 +24565,13 @@
     </row>
     <row r="389" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A389" s="7" t="s">
-        <v>1233</v>
+        <v>1232</v>
       </c>
       <c r="B389" s="7" t="s">
-        <v>1203</v>
+        <v>1202</v>
       </c>
       <c r="C389" s="7" t="s">
-        <v>1198</v>
+        <v>1197</v>
       </c>
       <c r="D389" s="7" t="s">
         <v>52</v>
@@ -24583,7 +24580,7 @@
         <v>19</v>
       </c>
       <c r="F389" s="9" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G389" s="8" t="s">
         <v>1062</v>
@@ -24619,13 +24616,13 @@
     </row>
     <row r="390" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A390" s="7" t="s">
-        <v>1206</v>
+        <v>1205</v>
       </c>
       <c r="B390" s="7" t="s">
-        <v>1205</v>
+        <v>1204</v>
       </c>
       <c r="C390" s="7" t="s">
-        <v>1204</v>
+        <v>1203</v>
       </c>
       <c r="D390" s="10" t="s">
         <v>921</v>
@@ -24670,13 +24667,13 @@
     </row>
     <row r="391" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A391" s="6" t="s">
-        <v>1234</v>
+        <v>1233</v>
       </c>
       <c r="B391" s="7" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="C391" s="7" t="s">
-        <v>1207</v>
+        <v>1206</v>
       </c>
       <c r="D391" s="7" t="s">
         <v>20</v>
@@ -24721,13 +24718,13 @@
     </row>
     <row r="392" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A392" s="6" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="B392" s="7" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="C392" s="7" t="s">
-        <v>1208</v>
+        <v>1207</v>
       </c>
       <c r="D392" s="7" t="s">
         <v>20</v>
@@ -24772,13 +24769,13 @@
     </row>
     <row r="393" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A393" s="6" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="B393" s="7" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="C393" s="7" t="s">
-        <v>1209</v>
+        <v>1208</v>
       </c>
       <c r="D393" s="7" t="s">
         <v>30</v>
@@ -24787,7 +24784,7 @@
         <v>19</v>
       </c>
       <c r="F393" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G393" s="7" t="s">
         <v>1062</v>
@@ -24823,13 +24820,13 @@
     </row>
     <row r="394" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A394" s="6" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="B394" s="7" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="C394" s="7" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="D394" s="7" t="s">
         <v>30</v>
@@ -24838,7 +24835,7 @@
         <v>19</v>
       </c>
       <c r="F394" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G394" s="7" t="s">
         <v>1062</v>
@@ -24874,13 +24871,13 @@
     </row>
     <row r="395" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A395" s="6" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="B395" s="7" t="s">
-        <v>1219</v>
+        <v>1218</v>
       </c>
       <c r="C395" s="7" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="D395" s="7" t="s">
         <v>30</v>
@@ -24889,10 +24886,10 @@
         <v>19</v>
       </c>
       <c r="F395" s="7" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="G395" s="7" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
       <c r="H395" s="7" t="s">
         <v>13</v>
@@ -24925,13 +24922,13 @@
     </row>
     <row r="396" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A396" s="6" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="B396" s="7" t="s">
-        <v>1220</v>
+        <v>1219</v>
       </c>
       <c r="C396" s="7" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="D396" s="7" t="s">
         <v>418</v>
@@ -24940,7 +24937,7 @@
         <v>19</v>
       </c>
       <c r="F396" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G396" s="7" t="s">
         <v>1062</v>
@@ -24976,13 +24973,13 @@
     </row>
     <row r="397" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A397" s="6" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
       <c r="B397" s="7" t="s">
-        <v>1221</v>
+        <v>1220</v>
       </c>
       <c r="C397" s="7" t="s">
-        <v>1213</v>
+        <v>1212</v>
       </c>
       <c r="D397" s="7" t="s">
         <v>418</v>
@@ -25027,13 +25024,13 @@
     </row>
     <row r="398" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A398" s="6" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="B398" s="7" t="s">
-        <v>1222</v>
+        <v>1221</v>
       </c>
       <c r="C398" s="7" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
       <c r="D398" s="7" t="s">
         <v>418</v>
@@ -25042,7 +25039,7 @@
         <v>19</v>
       </c>
       <c r="F398" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G398" s="7" t="s">
         <v>1062</v>
@@ -25078,13 +25075,13 @@
     </row>
     <row r="399" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A399" s="7" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="B399" s="7" t="s">
-        <v>1226</v>
+        <v>1225</v>
       </c>
       <c r="C399" s="7" t="s">
-        <v>1223</v>
+        <v>1222</v>
       </c>
       <c r="D399" s="7" t="s">
         <v>418</v>
@@ -25129,13 +25126,13 @@
     </row>
     <row r="400" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A400" s="7" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
       <c r="B400" s="7" t="s">
-        <v>1227</v>
+        <v>1226</v>
       </c>
       <c r="C400" s="7" t="s">
-        <v>1224</v>
+        <v>1223</v>
       </c>
       <c r="D400" s="7" t="s">
         <v>418</v>
@@ -25144,7 +25141,7 @@
         <v>19</v>
       </c>
       <c r="F400" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G400" s="7" t="s">
         <v>1062</v>
@@ -25180,13 +25177,13 @@
     </row>
     <row r="401" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A401" s="7" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="B401" s="7" t="s">
-        <v>1228</v>
+        <v>1227</v>
       </c>
       <c r="C401" s="7" t="s">
-        <v>1225</v>
+        <v>1224</v>
       </c>
       <c r="D401" s="7" t="s">
         <v>52</v>
@@ -25195,7 +25192,7 @@
         <v>19</v>
       </c>
       <c r="F401" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G401" s="8" t="s">
         <v>1062</v>
@@ -25231,13 +25228,13 @@
     </row>
     <row r="402" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A402" s="7" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="B402" s="7" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="C402" s="10" t="s">
-        <v>1245</v>
+        <v>1244</v>
       </c>
       <c r="D402" s="10" t="s">
         <v>701</v>
@@ -25246,7 +25243,7 @@
         <v>19</v>
       </c>
       <c r="F402" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G402" s="7" t="s">
         <v>1062</v>
@@ -25282,13 +25279,13 @@
     </row>
     <row r="403" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A403" s="11" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="B403" s="7" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="C403" s="10" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="D403" s="7" t="s">
         <v>127</v>
@@ -25297,7 +25294,7 @@
         <v>19</v>
       </c>
       <c r="F403" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G403" s="7" t="s">
         <v>1062</v>
@@ -25333,16 +25330,16 @@
     </row>
     <row r="404" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A404" s="6" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
       <c r="B404" s="7" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="C404" s="7" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="D404" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E404" s="8" t="s">
         <v>19</v>
@@ -25384,16 +25381,16 @@
     </row>
     <row r="405" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A405" s="6" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
       <c r="B405" s="7" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="C405" s="7" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="D405" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E405" s="8" t="s">
         <v>19</v>
@@ -25435,16 +25432,16 @@
     </row>
     <row r="406" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A406" s="6" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
       <c r="B406" s="7" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="C406" s="7" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="D406" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E406" s="8" t="s">
         <v>19</v>
@@ -25486,16 +25483,16 @@
     </row>
     <row r="407" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A407" s="6" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
       <c r="B407" s="7" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="C407" s="7" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="D407" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E407" s="8" t="s">
         <v>19</v>
@@ -25537,16 +25534,16 @@
     </row>
     <row r="408" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A408" s="6" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
       <c r="B408" s="7" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="C408" s="7" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="D408" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E408" s="8" t="s">
         <v>19</v>
@@ -25588,16 +25585,16 @@
     </row>
     <row r="409" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A409" s="6" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
       <c r="B409" s="7" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="C409" s="7" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="D409" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E409" s="8" t="s">
         <v>19</v>
@@ -25639,16 +25636,16 @@
     </row>
     <row r="410" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A410" s="6" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
       <c r="B410" s="7" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="C410" s="7" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="D410" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E410" s="8" t="s">
         <v>19</v>
@@ -25690,16 +25687,16 @@
     </row>
     <row r="411" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A411" s="6" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
       <c r="B411" s="7" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="C411" s="7" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="D411" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E411" s="8" t="s">
         <v>19</v>
@@ -25741,16 +25738,16 @@
     </row>
     <row r="412" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A412" s="6" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
       <c r="B412" s="7" t="s">
-        <v>1268</v>
+        <v>1267</v>
       </c>
       <c r="C412" s="7" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="D412" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E412" s="8" t="s">
         <v>19</v>
@@ -25792,16 +25789,16 @@
     </row>
     <row r="413" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A413" s="6" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
       <c r="B413" s="7" t="s">
-        <v>1270</v>
+        <v>1269</v>
       </c>
       <c r="C413" s="7" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="D413" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E413" s="8" t="s">
         <v>19</v>
@@ -25843,16 +25840,16 @@
     </row>
     <row r="414" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A414" s="6" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
       <c r="B414" s="7" t="s">
-        <v>1272</v>
+        <v>1271</v>
       </c>
       <c r="C414" s="7" t="s">
-        <v>1271</v>
+        <v>1270</v>
       </c>
       <c r="D414" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E414" s="8" t="s">
         <v>19</v>
@@ -25894,16 +25891,16 @@
     </row>
     <row r="415" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A415" s="6" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
       <c r="B415" s="7" t="s">
-        <v>1274</v>
+        <v>1273</v>
       </c>
       <c r="C415" s="7" t="s">
-        <v>1273</v>
+        <v>1272</v>
       </c>
       <c r="D415" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E415" s="8" t="s">
         <v>19</v>
@@ -25945,16 +25942,16 @@
     </row>
     <row r="416" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A416" s="6" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
       <c r="B416" s="7" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="C416" s="7" t="s">
-        <v>1275</v>
+        <v>1274</v>
       </c>
       <c r="D416" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E416" s="8" t="s">
         <v>19</v>
@@ -25996,16 +25993,16 @@
     </row>
     <row r="417" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A417" s="6" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
       <c r="B417" s="7" t="s">
-        <v>1278</v>
+        <v>1277</v>
       </c>
       <c r="C417" s="7" t="s">
-        <v>1277</v>
+        <v>1276</v>
       </c>
       <c r="D417" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E417" s="8" t="s">
         <v>19</v>
@@ -26047,16 +26044,16 @@
     </row>
     <row r="418" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A418" s="6" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
       <c r="B418" s="7" t="s">
-        <v>1280</v>
+        <v>1279</v>
       </c>
       <c r="C418" s="7" t="s">
-        <v>1279</v>
+        <v>1278</v>
       </c>
       <c r="D418" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E418" s="8" t="s">
         <v>19</v>
@@ -26098,16 +26095,16 @@
     </row>
     <row r="419" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A419" s="6" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
       <c r="B419" s="7" t="s">
-        <v>1282</v>
+        <v>1281</v>
       </c>
       <c r="C419" s="7" t="s">
-        <v>1281</v>
+        <v>1280</v>
       </c>
       <c r="D419" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E419" s="8" t="s">
         <v>19</v>
@@ -26149,16 +26146,16 @@
     </row>
     <row r="420" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A420" s="6" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
       <c r="B420" s="7" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="C420" s="7" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="D420" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E420" s="8" t="s">
         <v>19</v>
@@ -26200,16 +26197,16 @@
     </row>
     <row r="421" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A421" s="6" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="B421" s="7" t="s">
-        <v>1286</v>
+        <v>1285</v>
       </c>
       <c r="C421" s="7" t="s">
-        <v>1285</v>
+        <v>1284</v>
       </c>
       <c r="D421" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E421" s="8" t="s">
         <v>19</v>
@@ -26251,16 +26248,16 @@
     </row>
     <row r="422" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A422" s="6" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="B422" s="7" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="C422" s="7" t="s">
-        <v>1287</v>
+        <v>1286</v>
       </c>
       <c r="D422" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E422" s="8" t="s">
         <v>19</v>
@@ -26302,16 +26299,16 @@
     </row>
     <row r="423" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A423" s="6" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
       <c r="B423" s="7" t="s">
-        <v>1290</v>
+        <v>1289</v>
       </c>
       <c r="C423" s="7" t="s">
-        <v>1289</v>
+        <v>1288</v>
       </c>
       <c r="D423" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E423" s="8" t="s">
         <v>19</v>
@@ -26353,16 +26350,16 @@
     </row>
     <row r="424" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A424" s="6" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
       <c r="B424" s="7" t="s">
-        <v>1292</v>
+        <v>1291</v>
       </c>
       <c r="C424" s="7" t="s">
-        <v>1291</v>
+        <v>1290</v>
       </c>
       <c r="D424" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E424" s="8" t="s">
         <v>19</v>
@@ -26404,16 +26401,16 @@
     </row>
     <row r="425" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A425" s="6" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="B425" s="7" t="s">
-        <v>1294</v>
+        <v>1293</v>
       </c>
       <c r="C425" s="7" t="s">
-        <v>1293</v>
+        <v>1292</v>
       </c>
       <c r="D425" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E425" s="8" t="s">
         <v>19</v>
@@ -26455,16 +26452,16 @@
     </row>
     <row r="426" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A426" s="6" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
       <c r="B426" s="7" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="C426" s="7" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="D426" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E426" s="8" t="s">
         <v>19</v>
@@ -26506,16 +26503,16 @@
     </row>
     <row r="427" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A427" s="6" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
       <c r="B427" s="7" t="s">
-        <v>1298</v>
+        <v>1297</v>
       </c>
       <c r="C427" s="7" t="s">
-        <v>1297</v>
+        <v>1296</v>
       </c>
       <c r="D427" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E427" s="8" t="s">
         <v>19</v>
@@ -26557,16 +26554,16 @@
     </row>
     <row r="428" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A428" s="6" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
       <c r="B428" s="7" t="s">
-        <v>1300</v>
+        <v>1299</v>
       </c>
       <c r="C428" s="7" t="s">
-        <v>1299</v>
+        <v>1298</v>
       </c>
       <c r="D428" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E428" s="8" t="s">
         <v>19</v>
@@ -26608,16 +26605,16 @@
     </row>
     <row r="429" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A429" s="6" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
       <c r="B429" s="7" t="s">
-        <v>1302</v>
+        <v>1301</v>
       </c>
       <c r="C429" s="7" t="s">
-        <v>1301</v>
+        <v>1300</v>
       </c>
       <c r="D429" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E429" s="8" t="s">
         <v>19</v>
@@ -26659,16 +26656,16 @@
     </row>
     <row r="430" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A430" s="6" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="B430" s="7" t="s">
-        <v>1304</v>
+        <v>1303</v>
       </c>
       <c r="C430" s="7" t="s">
-        <v>1303</v>
+        <v>1302</v>
       </c>
       <c r="D430" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E430" s="8" t="s">
         <v>19</v>
@@ -26710,16 +26707,16 @@
     </row>
     <row r="431" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A431" s="6" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
       <c r="B431" s="7" t="s">
-        <v>1306</v>
+        <v>1305</v>
       </c>
       <c r="C431" s="7" t="s">
-        <v>1305</v>
+        <v>1304</v>
       </c>
       <c r="D431" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E431" s="8" t="s">
         <v>19</v>
@@ -26761,16 +26758,16 @@
     </row>
     <row r="432" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A432" s="6" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
       <c r="B432" s="7" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
       <c r="C432" s="7" t="s">
-        <v>1307</v>
+        <v>1306</v>
       </c>
       <c r="D432" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E432" s="8" t="s">
         <v>19</v>
@@ -26812,16 +26809,16 @@
     </row>
     <row r="433" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A433" s="6" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
       <c r="B433" s="7" t="s">
+        <v>1309</v>
+      </c>
+      <c r="C433" s="7" t="s">
+        <v>1308</v>
+      </c>
+      <c r="D433" s="7" t="s">
         <v>1310</v>
-      </c>
-      <c r="C433" s="7" t="s">
-        <v>1309</v>
-      </c>
-      <c r="D433" s="7" t="s">
-        <v>1311</v>
       </c>
       <c r="E433" s="8" t="s">
         <v>19</v>
@@ -26863,22 +26860,22 @@
     </row>
     <row r="434" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A434" s="7" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
       <c r="B434" s="7" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
       <c r="C434" s="7" t="s">
-        <v>1342</v>
+        <v>1341</v>
       </c>
       <c r="D434" s="7" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
       <c r="E434" s="8" t="s">
         <v>19</v>
       </c>
       <c r="F434" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G434" s="7" t="s">
         <v>1062</v>
@@ -26914,20 +26911,20 @@
     </row>
     <row r="435" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A435" s="7" t="s">
-        <v>1355</v>
+        <v>1354</v>
       </c>
       <c r="B435" s="7" t="s">
-        <v>1350</v>
+        <v>1349</v>
       </c>
       <c r="C435" s="10" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="D435" s="7"/>
       <c r="E435" s="8" t="s">
         <v>19</v>
       </c>
       <c r="F435" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G435" s="7" t="s">
         <v>1062</v>
@@ -26963,13 +26960,13 @@
     </row>
     <row r="436" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A436" s="7" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
       <c r="B436" s="7" t="s">
-        <v>1351</v>
+        <v>1350</v>
       </c>
       <c r="C436" s="10" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="D436" s="7"/>
       <c r="E436" s="8" t="s">
@@ -27012,20 +27009,20 @@
     </row>
     <row r="437" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A437" s="7" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="B437" s="7" t="s">
-        <v>1352</v>
+        <v>1351</v>
       </c>
       <c r="C437" s="10" t="s">
-        <v>1347</v>
+        <v>1346</v>
       </c>
       <c r="D437" s="7"/>
       <c r="E437" s="8" t="s">
         <v>19</v>
       </c>
       <c r="F437" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G437" s="7" t="s">
         <v>1062</v>
@@ -27061,20 +27058,20 @@
     </row>
     <row r="438" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A438" s="7" t="s">
-        <v>1358</v>
+        <v>1357</v>
       </c>
       <c r="B438" s="7" t="s">
-        <v>1353</v>
+        <v>1352</v>
       </c>
       <c r="C438" s="10" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
       <c r="D438" s="7"/>
       <c r="E438" s="8" t="s">
         <v>19</v>
       </c>
       <c r="F438" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G438" s="7" t="s">
         <v>1062</v>
@@ -27110,20 +27107,20 @@
     </row>
     <row r="439" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A439" s="7" t="s">
-        <v>1359</v>
+        <v>1358</v>
       </c>
       <c r="B439" s="7" t="s">
-        <v>1354</v>
+        <v>1353</v>
       </c>
       <c r="C439" s="10" t="s">
-        <v>1349</v>
+        <v>1348</v>
       </c>
       <c r="D439" s="7"/>
       <c r="E439" s="8" t="s">
         <v>19</v>
       </c>
       <c r="F439" s="7" t="s">
-        <v>1070</v>
+        <v>1069</v>
       </c>
       <c r="G439" s="7" t="s">
         <v>1062</v>
@@ -34286,31 +34283,32 @@
       <c r="T763" s="7"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:T439" xr:uid="{AF55B7BF-85DC-4082-9A73-200B4D79A598}"/>
   <conditionalFormatting sqref="A1:B1">
     <cfRule type="duplicateValues" dxfId="15" priority="23"/>
     <cfRule type="duplicateValues" dxfId="14" priority="24"/>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1">
-    <cfRule type="duplicateValues" dxfId="13" priority="37"/>
-    <cfRule type="duplicateValues" dxfId="12" priority="38"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="39"/>
-    <cfRule type="duplicateValues" dxfId="10" priority="40"/>
-  </conditionalFormatting>
   <conditionalFormatting sqref="C402">
-    <cfRule type="duplicateValues" dxfId="9" priority="8"/>
-    <cfRule type="duplicateValues" dxfId="8" priority="9"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="10"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="9"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C403">
-    <cfRule type="duplicateValues" dxfId="6" priority="5"/>
-    <cfRule type="duplicateValues" dxfId="5" priority="6"/>
-    <cfRule type="duplicateValues" dxfId="4" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="C435:C439">
-    <cfRule type="duplicateValues" dxfId="3" priority="1"/>
-    <cfRule type="duplicateValues" dxfId="2" priority="2"/>
-    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
-    <cfRule type="duplicateValues" dxfId="0" priority="4"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="4"/>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C1">
+    <cfRule type="duplicateValues" dxfId="3" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="42"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="43"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="44"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>